<commit_message>
Update tracker and add modules materials
</commit_message>
<xml_diff>
--- a/Halyna Maslak OTJ Tracker DE L5.xlsx
+++ b/Halyna Maslak OTJ Tracker DE L5.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29029"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DE Apprenticeship\Learning-Journal\Learning-Journal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{93A1D7F8-D132-4616-8B69-076B40A033A5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EF449FE1-61C9-4307-87C5-A333A807109D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="38640" windowHeight="21240" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="364" uniqueCount="288">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="385" uniqueCount="307">
   <si>
     <t xml:space="preserve">Apprenticeship Training Log </t>
   </si>
@@ -964,6 +964,63 @@
   </si>
   <si>
     <t>Google Cloud Professional Data Engineer Certification</t>
+  </si>
+  <si>
+    <t>Application of Statistics with Google</t>
+  </si>
+  <si>
+    <t>Google Hero in Data Management</t>
+  </si>
+  <si>
+    <t>End to End View of Data Products in GCP</t>
+  </si>
+  <si>
+    <t>Data Quality Uplift for Data Products</t>
+  </si>
+  <si>
+    <t>Building Data Products in GCP BigQuery</t>
+  </si>
+  <si>
+    <t>SQL OLAP and Windowing Functions</t>
+  </si>
+  <si>
+    <t>Shadowing: Data Engineering in Finance</t>
+  </si>
+  <si>
+    <t>K11, K10</t>
+  </si>
+  <si>
+    <t>S7</t>
+  </si>
+  <si>
+    <t>K11, K14</t>
+  </si>
+  <si>
+    <t>K4, K5, K9, K10</t>
+  </si>
+  <si>
+    <t>K10, K14</t>
+  </si>
+  <si>
+    <t>S9</t>
+  </si>
+  <si>
+    <t>K1, K2, K6, K8, K14, K17, K18, K20, K25</t>
+  </si>
+  <si>
+    <t>K14, K26, K29, S29, B6</t>
+  </si>
+  <si>
+    <t>Responsible AI</t>
+  </si>
+  <si>
+    <t>K29, S29</t>
+  </si>
+  <si>
+    <t>What Not to Do: Data Storytelling</t>
+  </si>
+  <si>
+    <t>K30</t>
   </si>
 </sst>
 </file>
@@ -2054,7 +2111,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="9" fontId="29" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="206">
+  <cellXfs count="209">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
@@ -2321,42 +2378,11 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2366,12 +2392,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
@@ -2412,6 +2432,61 @@
     <xf numFmtId="0" fontId="15" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="25" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="0" borderId="19" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="17" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
@@ -2433,24 +2508,6 @@
     <xf numFmtId="0" fontId="16" fillId="0" borderId="41" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2463,6 +2520,9 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -2877,7 +2937,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP313"/>
+  <dimension ref="A1:AP315"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -2940,12 +3000,12 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="168"/>
-      <c r="K2" s="169"/>
-      <c r="L2" s="169"/>
-      <c r="M2" s="169"/>
-      <c r="N2" s="169"/>
-      <c r="O2" s="170"/>
+      <c r="J2" s="176"/>
+      <c r="K2" s="177"/>
+      <c r="L2" s="177"/>
+      <c r="M2" s="177"/>
+      <c r="N2" s="177"/>
+      <c r="O2" s="178"/>
       <c r="P2" s="37"/>
       <c r="Q2" s="37"/>
       <c r="R2" s="2"/>
@@ -2976,14 +3036,14 @@
     </row>
     <row r="3" spans="1:42" ht="220.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
-      <c r="B3" s="174" t="s">
+      <c r="B3" s="158" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="174"/>
-      <c r="D3" s="174"/>
-      <c r="E3" s="174"/>
-      <c r="F3" s="174"/>
-      <c r="G3" s="175"/>
+      <c r="C3" s="158"/>
+      <c r="D3" s="158"/>
+      <c r="E3" s="158"/>
+      <c r="F3" s="158"/>
+      <c r="G3" s="159"/>
       <c r="H3" s="1"/>
       <c r="I3" s="2"/>
       <c r="J3" s="54"/>
@@ -3081,14 +3141,14 @@
       <c r="G5" s="57" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="188"/>
+      <c r="H5" s="175"/>
       <c r="I5" s="2"/>
-      <c r="J5" s="171"/>
-      <c r="K5" s="172"/>
-      <c r="L5" s="172"/>
-      <c r="M5" s="172"/>
-      <c r="N5" s="172"/>
-      <c r="O5" s="173"/>
+      <c r="J5" s="160"/>
+      <c r="K5" s="161"/>
+      <c r="L5" s="161"/>
+      <c r="M5" s="161"/>
+      <c r="N5" s="161"/>
+      <c r="O5" s="162"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
@@ -3136,7 +3196,7 @@
         <f t="shared" ref="G6:G18" si="0">IF(NOT(ISBLANK(D6)), SUM(E6:F6), 0)</f>
         <v>6</v>
       </c>
-      <c r="H6" s="188"/>
+      <c r="H6" s="175"/>
       <c r="I6" s="2"/>
       <c r="J6" s="143"/>
       <c r="K6" s="143"/>
@@ -3191,7 +3251,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="H7" s="188"/>
+      <c r="H7" s="175"/>
       <c r="I7" s="4"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
@@ -3246,7 +3306,7 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="H8" s="188"/>
+      <c r="H8" s="175"/>
       <c r="I8" s="4"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
@@ -3301,7 +3361,7 @@
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="H9" s="188"/>
+      <c r="H9" s="175"/>
       <c r="I9" s="4"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
@@ -3343,7 +3403,9 @@
         <v>12</v>
       </c>
       <c r="C10" s="58"/>
-      <c r="D10" s="58"/>
+      <c r="D10" s="81">
+        <v>45826</v>
+      </c>
       <c r="E10" s="58">
         <v>12</v>
       </c>
@@ -3352,9 +3414,9 @@
       </c>
       <c r="G10" s="138">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H10" s="188"/>
+        <v>24</v>
+      </c>
+      <c r="H10" s="175"/>
       <c r="I10" s="4"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
@@ -3396,7 +3458,9 @@
         <v>13</v>
       </c>
       <c r="C11" s="58"/>
-      <c r="D11" s="58"/>
+      <c r="D11" s="81">
+        <v>45875</v>
+      </c>
       <c r="E11" s="58">
         <v>24</v>
       </c>
@@ -3405,9 +3469,9 @@
       </c>
       <c r="G11" s="138">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H11" s="188"/>
+        <v>46</v>
+      </c>
+      <c r="H11" s="175"/>
       <c r="I11" s="4"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
@@ -3460,7 +3524,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H12" s="188"/>
+      <c r="H12" s="175"/>
       <c r="I12" s="4"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
@@ -3513,7 +3577,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H13" s="188"/>
+      <c r="H13" s="175"/>
       <c r="I13" s="4"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
@@ -3566,7 +3630,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H14" s="188"/>
+      <c r="H14" s="175"/>
       <c r="I14" s="4"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
@@ -3619,7 +3683,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H15" s="188"/>
+      <c r="H15" s="175"/>
       <c r="I15" s="4"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
@@ -3672,7 +3736,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H16" s="188"/>
+      <c r="H16" s="175"/>
       <c r="I16" s="4"/>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
@@ -3725,14 +3789,14 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H17" s="188"/>
+      <c r="H17" s="175"/>
       <c r="I17" s="4"/>
-      <c r="J17" s="171"/>
-      <c r="K17" s="172"/>
-      <c r="L17" s="172"/>
-      <c r="M17" s="172"/>
-      <c r="N17" s="172"/>
-      <c r="O17" s="173"/>
+      <c r="J17" s="160"/>
+      <c r="K17" s="161"/>
+      <c r="L17" s="161"/>
+      <c r="M17" s="161"/>
+      <c r="N17" s="161"/>
+      <c r="O17" s="162"/>
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
       <c r="R17" s="2"/>
@@ -3778,7 +3842,7 @@
         <f t="shared" si="0"/>
         <v>0</v>
       </c>
-      <c r="H18" s="188"/>
+      <c r="H18" s="175"/>
       <c r="I18" s="4"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
@@ -3831,9 +3895,9 @@
       </c>
       <c r="G19" s="142">
         <f>SUM(G6:G18)</f>
-        <v>116</v>
-      </c>
-      <c r="H19" s="188"/>
+        <v>186</v>
+      </c>
+      <c r="H19" s="175"/>
       <c r="I19" s="4"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
@@ -3985,14 +4049,14 @@
         <f>IF(NOT(ISBLANK(D22)), SUM(E22:F22), 0)</f>
         <v>24</v>
       </c>
-      <c r="H22" s="159"/>
+      <c r="H22" s="184"/>
       <c r="I22" s="2"/>
-      <c r="J22" s="171"/>
-      <c r="K22" s="172"/>
-      <c r="L22" s="172"/>
-      <c r="M22" s="172"/>
-      <c r="N22" s="172"/>
-      <c r="O22" s="173"/>
+      <c r="J22" s="160"/>
+      <c r="K22" s="161"/>
+      <c r="L22" s="161"/>
+      <c r="M22" s="161"/>
+      <c r="N22" s="161"/>
+      <c r="O22" s="162"/>
       <c r="P22" s="2"/>
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
@@ -4036,7 +4100,7 @@
         <f>IF(NOT(ISBLANK(D23)), SUM(E23:F23), 0)</f>
         <v>0</v>
       </c>
-      <c r="H23" s="159"/>
+      <c r="H23" s="184"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
@@ -4087,7 +4151,7 @@
         <f>IF(NOT(ISBLANK(D24)), SUM(E24:F24), 0)</f>
         <v>0</v>
       </c>
-      <c r="H24" s="159"/>
+      <c r="H24" s="184"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -4138,7 +4202,7 @@
         <f>IF(NOT(ISBLANK(D25)), SUM(E25:F25), 0)</f>
         <v>0</v>
       </c>
-      <c r="H25" s="159"/>
+      <c r="H25" s="184"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -4189,7 +4253,7 @@
         <f>IF(NOT(ISBLANK(D26)), SUM(E26:F26), 0)</f>
         <v>0</v>
       </c>
-      <c r="H26" s="159"/>
+      <c r="H26" s="184"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
@@ -4233,7 +4297,7 @@
       <c r="E27" s="58"/>
       <c r="F27" s="58"/>
       <c r="G27" s="58"/>
-      <c r="H27" s="159"/>
+      <c r="H27" s="184"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
@@ -4288,7 +4352,7 @@
         <f>SUM(G22:H27)</f>
         <v>24</v>
       </c>
-      <c r="H28" s="159"/>
+      <c r="H28" s="184"/>
       <c r="I28" s="4"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
@@ -4326,20 +4390,20 @@
     </row>
     <row r="29" spans="1:42" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="182"/>
-      <c r="C29" s="183"/>
-      <c r="D29" s="183"/>
-      <c r="E29" s="183"/>
-      <c r="F29" s="183"/>
-      <c r="G29" s="183"/>
-      <c r="H29" s="184"/>
+      <c r="B29" s="169"/>
+      <c r="C29" s="170"/>
+      <c r="D29" s="170"/>
+      <c r="E29" s="170"/>
+      <c r="F29" s="170"/>
+      <c r="G29" s="170"/>
+      <c r="H29" s="171"/>
       <c r="I29" s="2"/>
-      <c r="J29" s="171"/>
-      <c r="K29" s="172"/>
-      <c r="L29" s="172"/>
-      <c r="M29" s="172"/>
-      <c r="N29" s="172"/>
-      <c r="O29" s="173"/>
+      <c r="J29" s="160"/>
+      <c r="K29" s="161"/>
+      <c r="L29" s="161"/>
+      <c r="M29" s="161"/>
+      <c r="N29" s="161"/>
+      <c r="O29" s="162"/>
       <c r="P29" s="2"/>
       <c r="Q29" s="2"/>
       <c r="R29" s="2"/>
@@ -4377,12 +4441,12 @@
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
-      <c r="J30" s="179"/>
-      <c r="K30" s="180"/>
-      <c r="L30" s="180"/>
-      <c r="M30" s="180"/>
-      <c r="N30" s="180"/>
-      <c r="O30" s="181"/>
+      <c r="J30" s="166"/>
+      <c r="K30" s="167"/>
+      <c r="L30" s="167"/>
+      <c r="M30" s="167"/>
+      <c r="N30" s="167"/>
+      <c r="O30" s="168"/>
       <c r="P30" s="2"/>
       <c r="Q30" s="2"/>
       <c r="R30" s="2"/>
@@ -4413,13 +4477,13 @@
     </row>
     <row r="31" spans="1:42" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
-      <c r="B31" s="185" t="s">
+      <c r="B31" s="172" t="s">
         <v>33</v>
       </c>
-      <c r="C31" s="186"/>
-      <c r="D31" s="186"/>
-      <c r="E31" s="186"/>
-      <c r="F31" s="187"/>
+      <c r="C31" s="173"/>
+      <c r="D31" s="173"/>
+      <c r="E31" s="173"/>
+      <c r="F31" s="174"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
@@ -4599,23 +4663,23 @@
       <c r="D35" s="64" t="s">
         <v>37</v>
       </c>
-      <c r="E35" s="164" t="s">
+      <c r="E35" s="180" t="s">
         <v>38</v>
       </c>
-      <c r="F35" s="164"/>
+      <c r="F35" s="180"/>
       <c r="G35" s="64" t="s">
         <v>25</v>
       </c>
-      <c r="H35" s="160" t="s">
+      <c r="H35" s="185" t="s">
         <v>39</v>
       </c>
       <c r="I35" s="4"/>
-      <c r="J35" s="171"/>
-      <c r="K35" s="172"/>
-      <c r="L35" s="172"/>
-      <c r="M35" s="172"/>
-      <c r="N35" s="172"/>
-      <c r="O35" s="173"/>
+      <c r="J35" s="160"/>
+      <c r="K35" s="161"/>
+      <c r="L35" s="161"/>
+      <c r="M35" s="161"/>
+      <c r="N35" s="161"/>
+      <c r="O35" s="162"/>
       <c r="P35" s="2"/>
       <c r="Q35" s="2"/>
       <c r="R35" s="2"/>
@@ -4655,14 +4719,14 @@
       <c r="D36" s="152">
         <v>45694</v>
       </c>
-      <c r="E36" s="165" t="s">
+      <c r="E36" s="181" t="s">
         <v>263</v>
       </c>
-      <c r="F36" s="166"/>
+      <c r="F36" s="182"/>
       <c r="G36" s="106">
         <v>0.5</v>
       </c>
-      <c r="H36" s="161"/>
+      <c r="H36" s="186"/>
       <c r="I36" s="4"/>
       <c r="J36" s="2"/>
       <c r="K36" s="2"/>
@@ -4709,21 +4773,21 @@
       <c r="D37" s="153">
         <v>45699</v>
       </c>
-      <c r="E37" s="165" t="s">
+      <c r="E37" s="181" t="s">
         <v>263</v>
       </c>
-      <c r="F37" s="166"/>
+      <c r="F37" s="182"/>
       <c r="G37" s="106">
         <v>2</v>
       </c>
-      <c r="H37" s="161"/>
+      <c r="H37" s="186"/>
       <c r="I37" s="5"/>
-      <c r="J37" s="176"/>
-      <c r="K37" s="177"/>
-      <c r="L37" s="177"/>
-      <c r="M37" s="177"/>
-      <c r="N37" s="177"/>
-      <c r="O37" s="178"/>
+      <c r="J37" s="163"/>
+      <c r="K37" s="164"/>
+      <c r="L37" s="164"/>
+      <c r="M37" s="164"/>
+      <c r="N37" s="164"/>
+      <c r="O37" s="165"/>
       <c r="P37" s="2"/>
       <c r="Q37" s="2"/>
       <c r="R37" s="2"/>
@@ -4763,14 +4827,14 @@
       <c r="D38" s="153">
         <v>45701</v>
       </c>
-      <c r="E38" s="167" t="s">
+      <c r="E38" s="183" t="s">
         <v>280</v>
       </c>
-      <c r="F38" s="166"/>
+      <c r="F38" s="182"/>
       <c r="G38" s="106">
         <v>7</v>
       </c>
-      <c r="H38" s="161"/>
+      <c r="H38" s="186"/>
       <c r="I38" s="2"/>
       <c r="J38" s="156"/>
       <c r="K38" s="156"/>
@@ -4817,14 +4881,14 @@
       <c r="D39" s="154">
         <v>45712</v>
       </c>
-      <c r="E39" s="158" t="s">
+      <c r="E39" s="179" t="s">
         <v>268</v>
       </c>
-      <c r="F39" s="158"/>
+      <c r="F39" s="179"/>
       <c r="G39" s="106">
         <v>0.5</v>
       </c>
-      <c r="H39" s="161"/>
+      <c r="H39" s="186"/>
       <c r="I39" s="2"/>
       <c r="J39" s="2"/>
       <c r="K39" s="2"/>
@@ -4871,21 +4935,21 @@
       <c r="D40" s="154">
         <v>45712</v>
       </c>
-      <c r="E40" s="158" t="s">
+      <c r="E40" s="179" t="s">
         <v>263</v>
       </c>
-      <c r="F40" s="158"/>
+      <c r="F40" s="179"/>
       <c r="G40" s="106">
         <v>0.5</v>
       </c>
-      <c r="H40" s="161"/>
+      <c r="H40" s="186"/>
       <c r="I40" s="2"/>
-      <c r="J40" s="171"/>
-      <c r="K40" s="172"/>
-      <c r="L40" s="172"/>
-      <c r="M40" s="172"/>
-      <c r="N40" s="172"/>
-      <c r="O40" s="173"/>
+      <c r="J40" s="160"/>
+      <c r="K40" s="161"/>
+      <c r="L40" s="161"/>
+      <c r="M40" s="161"/>
+      <c r="N40" s="161"/>
+      <c r="O40" s="162"/>
       <c r="P40" s="2"/>
       <c r="Q40" s="2"/>
       <c r="R40" s="2"/>
@@ -4925,14 +4989,14 @@
       <c r="D41" s="154">
         <v>45712</v>
       </c>
-      <c r="E41" s="158" t="s">
+      <c r="E41" s="179" t="s">
         <v>269</v>
       </c>
-      <c r="F41" s="158"/>
+      <c r="F41" s="179"/>
       <c r="G41" s="106">
         <v>0.5</v>
       </c>
-      <c r="H41" s="161"/>
+      <c r="H41" s="186"/>
       <c r="I41" s="2"/>
       <c r="J41" s="2"/>
       <c r="K41" s="2"/>
@@ -4979,14 +5043,14 @@
       <c r="D42" s="154">
         <v>45713</v>
       </c>
-      <c r="E42" s="158" t="s">
+      <c r="E42" s="179" t="s">
         <v>271</v>
       </c>
-      <c r="F42" s="158"/>
+      <c r="F42" s="179"/>
       <c r="G42" s="106">
         <v>0.5</v>
       </c>
-      <c r="H42" s="161"/>
+      <c r="H42" s="186"/>
       <c r="I42" s="2"/>
       <c r="J42" s="2"/>
       <c r="K42" s="2"/>
@@ -5033,14 +5097,14 @@
       <c r="D43" s="154">
         <v>45713</v>
       </c>
-      <c r="E43" s="158" t="s">
+      <c r="E43" s="179" t="s">
         <v>273</v>
       </c>
-      <c r="F43" s="158"/>
+      <c r="F43" s="179"/>
       <c r="G43" s="106">
         <v>0.5</v>
       </c>
-      <c r="H43" s="161"/>
+      <c r="H43" s="186"/>
       <c r="I43" s="2"/>
       <c r="J43" s="2"/>
       <c r="K43" s="2"/>
@@ -5087,14 +5151,14 @@
       <c r="D44" s="154">
         <v>45713</v>
       </c>
-      <c r="E44" s="158" t="s">
+      <c r="E44" s="179" t="s">
         <v>271</v>
       </c>
-      <c r="F44" s="158"/>
+      <c r="F44" s="179"/>
       <c r="G44" s="106">
         <v>0.5</v>
       </c>
-      <c r="H44" s="161"/>
+      <c r="H44" s="186"/>
       <c r="I44" s="2"/>
       <c r="J44" s="2"/>
       <c r="K44" s="2"/>
@@ -5141,14 +5205,14 @@
       <c r="D45" s="154">
         <v>45803</v>
       </c>
-      <c r="E45" s="158" t="s">
+      <c r="E45" s="179" t="s">
         <v>276</v>
       </c>
-      <c r="F45" s="158"/>
+      <c r="F45" s="179"/>
       <c r="G45" s="149">
         <v>0.5</v>
       </c>
-      <c r="H45" s="161"/>
+      <c r="H45" s="186"/>
       <c r="I45" s="2"/>
       <c r="J45" s="2"/>
       <c r="K45" s="2"/>
@@ -5195,14 +5259,14 @@
       <c r="D46" s="154">
         <v>45714</v>
       </c>
-      <c r="E46" s="158" t="s">
+      <c r="E46" s="179" t="s">
         <v>271</v>
       </c>
-      <c r="F46" s="158"/>
+      <c r="F46" s="179"/>
       <c r="G46" s="106">
         <v>0.5</v>
       </c>
-      <c r="H46" s="161"/>
+      <c r="H46" s="186"/>
       <c r="I46" s="2"/>
       <c r="J46" s="2"/>
       <c r="K46" s="2"/>
@@ -5249,14 +5313,14 @@
       <c r="D47" s="154">
         <v>45723</v>
       </c>
-      <c r="E47" s="158" t="s">
+      <c r="E47" s="179" t="s">
         <v>271</v>
       </c>
-      <c r="F47" s="158"/>
+      <c r="F47" s="179"/>
       <c r="G47" s="106">
         <v>1</v>
       </c>
-      <c r="H47" s="161"/>
+      <c r="H47" s="186"/>
       <c r="I47" s="2"/>
       <c r="J47" s="2"/>
       <c r="K47" s="2"/>
@@ -5301,14 +5365,14 @@
       <c r="D48" s="81">
         <v>45726</v>
       </c>
-      <c r="E48" s="158" t="s">
+      <c r="E48" s="179" t="s">
         <v>282</v>
       </c>
-      <c r="F48" s="158"/>
+      <c r="F48" s="179"/>
       <c r="G48" s="106">
         <v>0.5</v>
       </c>
-      <c r="H48" s="161"/>
+      <c r="H48" s="186"/>
       <c r="I48" s="43"/>
       <c r="J48" s="37"/>
       <c r="K48" s="2"/>
@@ -5353,14 +5417,14 @@
       <c r="D49" s="81">
         <v>45743</v>
       </c>
-      <c r="E49" s="158" t="s">
+      <c r="E49" s="179" t="s">
         <v>284</v>
       </c>
-      <c r="F49" s="158"/>
+      <c r="F49" s="179"/>
       <c r="G49" s="63">
         <v>2</v>
       </c>
-      <c r="H49" s="161"/>
+      <c r="H49" s="186"/>
       <c r="I49" s="43"/>
       <c r="J49" s="37"/>
       <c r="K49" s="2"/>
@@ -5407,12 +5471,14 @@
       <c r="D50" s="81">
         <v>45805</v>
       </c>
-      <c r="E50" s="158"/>
-      <c r="F50" s="158"/>
+      <c r="E50" s="179" t="s">
+        <v>271</v>
+      </c>
+      <c r="F50" s="179"/>
       <c r="G50" s="63">
         <v>1</v>
       </c>
-      <c r="H50" s="161"/>
+      <c r="H50" s="186"/>
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
@@ -5457,12 +5523,14 @@
       <c r="D51" s="81">
         <v>45806</v>
       </c>
-      <c r="E51" s="158"/>
-      <c r="F51" s="158"/>
+      <c r="E51" s="179" t="s">
+        <v>295</v>
+      </c>
+      <c r="F51" s="179"/>
       <c r="G51" s="63">
         <v>1</v>
       </c>
-      <c r="H51" s="161"/>
+      <c r="H51" s="186"/>
       <c r="I51" s="2"/>
       <c r="J51" s="2"/>
       <c r="K51" s="2"/>
@@ -5507,12 +5575,14 @@
       <c r="D52" s="81">
         <v>45793</v>
       </c>
-      <c r="E52" s="158"/>
-      <c r="F52" s="158"/>
+      <c r="E52" s="179" t="s">
+        <v>302</v>
+      </c>
+      <c r="F52" s="179"/>
       <c r="G52" s="63">
         <v>30</v>
       </c>
-      <c r="H52" s="161"/>
+      <c r="H52" s="186"/>
       <c r="I52" s="2"/>
       <c r="J52" s="2"/>
       <c r="K52" s="2"/>
@@ -5550,13 +5620,21 @@
     </row>
     <row r="53" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="3"/>
-      <c r="B53" s="79"/>
+      <c r="B53" s="79" t="s">
+        <v>288</v>
+      </c>
       <c r="C53" s="78"/>
-      <c r="D53" s="58"/>
-      <c r="E53" s="158"/>
-      <c r="F53" s="158"/>
-      <c r="G53" s="63"/>
-      <c r="H53" s="161"/>
+      <c r="D53" s="81">
+        <v>45855</v>
+      </c>
+      <c r="E53" s="179" t="s">
+        <v>296</v>
+      </c>
+      <c r="F53" s="179"/>
+      <c r="G53" s="63">
+        <v>1</v>
+      </c>
+      <c r="H53" s="186"/>
       <c r="I53" s="2"/>
       <c r="J53" s="2"/>
       <c r="K53" s="2"/>
@@ -5594,13 +5672,21 @@
     </row>
     <row r="54" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A54" s="3"/>
-      <c r="B54" s="79"/>
+      <c r="B54" s="79" t="s">
+        <v>303</v>
+      </c>
       <c r="C54" s="78"/>
-      <c r="D54" s="58"/>
-      <c r="E54" s="158"/>
-      <c r="F54" s="158"/>
-      <c r="G54" s="63"/>
-      <c r="H54" s="161"/>
+      <c r="D54" s="81">
+        <v>45859</v>
+      </c>
+      <c r="E54" s="207" t="s">
+        <v>304</v>
+      </c>
+      <c r="F54" s="208"/>
+      <c r="G54" s="63">
+        <v>1</v>
+      </c>
+      <c r="H54" s="186"/>
       <c r="I54" s="2"/>
       <c r="J54" s="2"/>
       <c r="K54" s="2"/>
@@ -5638,13 +5724,21 @@
     </row>
     <row r="55" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A55" s="3"/>
-      <c r="B55" s="79"/>
+      <c r="B55" s="79" t="s">
+        <v>305</v>
+      </c>
       <c r="C55" s="78"/>
-      <c r="D55" s="58"/>
-      <c r="E55" s="158"/>
-      <c r="F55" s="158"/>
-      <c r="G55" s="63"/>
-      <c r="H55" s="161"/>
+      <c r="D55" s="81">
+        <v>45866</v>
+      </c>
+      <c r="E55" s="207" t="s">
+        <v>306</v>
+      </c>
+      <c r="F55" s="208"/>
+      <c r="G55" s="63">
+        <v>1</v>
+      </c>
+      <c r="H55" s="186"/>
       <c r="I55" s="2"/>
       <c r="J55" s="2"/>
       <c r="K55" s="2"/>
@@ -5682,13 +5776,21 @@
     </row>
     <row r="56" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A56" s="3"/>
-      <c r="B56" s="58"/>
+      <c r="B56" s="79" t="s">
+        <v>289</v>
+      </c>
       <c r="C56" s="78"/>
-      <c r="D56" s="58"/>
-      <c r="E56" s="158"/>
-      <c r="F56" s="158"/>
-      <c r="G56" s="63"/>
-      <c r="H56" s="161"/>
+      <c r="D56" s="81">
+        <v>45873</v>
+      </c>
+      <c r="E56" s="179" t="s">
+        <v>297</v>
+      </c>
+      <c r="F56" s="179"/>
+      <c r="G56" s="63">
+        <v>1</v>
+      </c>
+      <c r="H56" s="186"/>
       <c r="I56" s="2"/>
       <c r="J56" s="2"/>
       <c r="K56" s="2"/>
@@ -5726,13 +5828,21 @@
     </row>
     <row r="57" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A57" s="3"/>
-      <c r="B57" s="58"/>
+      <c r="B57" s="79" t="s">
+        <v>290</v>
+      </c>
       <c r="C57" s="78"/>
-      <c r="D57" s="58"/>
-      <c r="E57" s="158"/>
-      <c r="F57" s="158"/>
-      <c r="G57" s="63"/>
-      <c r="H57" s="161"/>
+      <c r="D57" s="81">
+        <v>45873</v>
+      </c>
+      <c r="E57" s="179" t="s">
+        <v>297</v>
+      </c>
+      <c r="F57" s="179"/>
+      <c r="G57" s="63">
+        <v>0.5</v>
+      </c>
+      <c r="H57" s="186"/>
       <c r="I57" s="2"/>
       <c r="J57" s="2"/>
       <c r="K57" s="2"/>
@@ -5770,13 +5880,21 @@
     </row>
     <row r="58" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
-      <c r="B58" s="58"/>
+      <c r="B58" s="58" t="s">
+        <v>291</v>
+      </c>
       <c r="C58" s="78"/>
-      <c r="D58" s="58"/>
-      <c r="E58" s="158"/>
-      <c r="F58" s="158"/>
-      <c r="G58" s="63"/>
-      <c r="H58" s="161"/>
+      <c r="D58" s="81">
+        <v>45874</v>
+      </c>
+      <c r="E58" s="179" t="s">
+        <v>298</v>
+      </c>
+      <c r="F58" s="179"/>
+      <c r="G58" s="63">
+        <v>1</v>
+      </c>
+      <c r="H58" s="186"/>
       <c r="I58" s="2"/>
       <c r="J58" s="2"/>
       <c r="K58" s="2"/>
@@ -5814,13 +5932,21 @@
     </row>
     <row r="59" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
-      <c r="B59" s="58"/>
+      <c r="B59" s="58" t="s">
+        <v>292</v>
+      </c>
       <c r="C59" s="78"/>
-      <c r="D59" s="58"/>
-      <c r="E59" s="158"/>
-      <c r="F59" s="158"/>
-      <c r="G59" s="63"/>
-      <c r="H59" s="161"/>
+      <c r="D59" s="81">
+        <v>45880</v>
+      </c>
+      <c r="E59" s="179" t="s">
+        <v>299</v>
+      </c>
+      <c r="F59" s="179"/>
+      <c r="G59" s="63">
+        <v>0.5</v>
+      </c>
+      <c r="H59" s="186"/>
       <c r="I59" s="2"/>
       <c r="J59" s="2"/>
       <c r="K59" s="2"/>
@@ -5858,13 +5984,21 @@
     </row>
     <row r="60" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
-      <c r="B60" s="58"/>
+      <c r="B60" s="58" t="s">
+        <v>293</v>
+      </c>
       <c r="C60" s="78"/>
-      <c r="D60" s="58"/>
-      <c r="E60" s="158"/>
-      <c r="F60" s="158"/>
-      <c r="G60" s="63"/>
-      <c r="H60" s="161"/>
+      <c r="D60" s="81">
+        <v>45884</v>
+      </c>
+      <c r="E60" s="179" t="s">
+        <v>300</v>
+      </c>
+      <c r="F60" s="179"/>
+      <c r="G60" s="63">
+        <v>1</v>
+      </c>
+      <c r="H60" s="186"/>
       <c r="I60" s="2"/>
       <c r="J60" s="2"/>
       <c r="K60" s="2"/>
@@ -5902,13 +6036,21 @@
     </row>
     <row r="61" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3"/>
-      <c r="B61" s="58"/>
+      <c r="B61" s="58" t="s">
+        <v>294</v>
+      </c>
       <c r="C61" s="78"/>
-      <c r="D61" s="58"/>
-      <c r="E61" s="158"/>
-      <c r="F61" s="158"/>
-      <c r="G61" s="63"/>
-      <c r="H61" s="161"/>
+      <c r="D61" s="81">
+        <v>45888</v>
+      </c>
+      <c r="E61" s="206" t="s">
+        <v>301</v>
+      </c>
+      <c r="F61" s="206"/>
+      <c r="G61" s="63">
+        <v>7</v>
+      </c>
+      <c r="H61" s="186"/>
       <c r="I61" s="2"/>
       <c r="J61" s="2"/>
       <c r="K61" s="2"/>
@@ -5944,20 +6086,15 @@
       <c r="AO61" s="2"/>
       <c r="AP61" s="2"/>
     </row>
-    <row r="62" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3"/>
-      <c r="B62" s="129" t="s">
-        <v>7</v>
-      </c>
-      <c r="C62" s="130"/>
-      <c r="D62" s="131"/>
-      <c r="E62" s="163"/>
-      <c r="F62" s="163"/>
-      <c r="G62" s="36">
-        <f>SUM(G36:G61)</f>
-        <v>49</v>
-      </c>
-      <c r="H62" s="162"/>
+      <c r="B62" s="58"/>
+      <c r="C62" s="78"/>
+      <c r="D62" s="58"/>
+      <c r="E62" s="179"/>
+      <c r="F62" s="179"/>
+      <c r="G62" s="63"/>
+      <c r="H62" s="186"/>
       <c r="I62" s="2"/>
       <c r="J62" s="2"/>
       <c r="K62" s="2"/>
@@ -5993,15 +6130,15 @@
       <c r="AO62" s="2"/>
       <c r="AP62" s="2"/>
     </row>
-    <row r="63" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3"/>
-      <c r="B63" s="136"/>
-      <c r="C63" s="132"/>
-      <c r="D63" s="133"/>
-      <c r="E63" s="1"/>
-      <c r="F63" s="1"/>
-      <c r="G63" s="137"/>
-      <c r="H63" s="128"/>
+      <c r="B63" s="58"/>
+      <c r="C63" s="78"/>
+      <c r="D63" s="58"/>
+      <c r="E63" s="179"/>
+      <c r="F63" s="179"/>
+      <c r="G63" s="63"/>
+      <c r="H63" s="186"/>
       <c r="I63" s="2"/>
       <c r="J63" s="2"/>
       <c r="K63" s="2"/>
@@ -6037,20 +6174,20 @@
       <c r="AO63" s="2"/>
       <c r="AP63" s="2"/>
     </row>
-    <row r="64" spans="1:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A64" s="3"/>
-      <c r="B64" s="134" t="s">
-        <v>40</v>
-      </c>
-      <c r="C64" s="134"/>
-      <c r="D64" s="135"/>
-      <c r="E64" s="27"/>
-      <c r="F64" s="27"/>
-      <c r="G64" s="51">
-        <f>G62+G19+G28+G63</f>
-        <v>189</v>
-      </c>
-      <c r="H64" s="44"/>
+      <c r="B64" s="129" t="s">
+        <v>7</v>
+      </c>
+      <c r="C64" s="130"/>
+      <c r="D64" s="131"/>
+      <c r="E64" s="188"/>
+      <c r="F64" s="188"/>
+      <c r="G64" s="36">
+        <f>SUM(G36:G63)</f>
+        <v>63</v>
+      </c>
+      <c r="H64" s="187"/>
       <c r="I64" s="2"/>
       <c r="J64" s="2"/>
       <c r="K64" s="2"/>
@@ -6088,13 +6225,13 @@
     </row>
     <row r="65" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A65" s="3"/>
-      <c r="B65" s="2"/>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
-      <c r="G65" s="2"/>
-      <c r="H65" s="43"/>
+      <c r="B65" s="136"/>
+      <c r="C65" s="132"/>
+      <c r="D65" s="133"/>
+      <c r="E65" s="1"/>
+      <c r="F65" s="1"/>
+      <c r="G65" s="137"/>
+      <c r="H65" s="128"/>
       <c r="I65" s="2"/>
       <c r="J65" s="2"/>
       <c r="K65" s="2"/>
@@ -6130,13 +6267,20 @@
       <c r="AO65" s="2"/>
       <c r="AP65" s="2"/>
     </row>
-    <row r="66" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A66" s="3"/>
-      <c r="B66" s="1"/>
-      <c r="D66" s="2"/>
-      <c r="F66" s="2"/>
-      <c r="G66" s="2"/>
-      <c r="H66" s="37"/>
+      <c r="B66" s="134" t="s">
+        <v>40</v>
+      </c>
+      <c r="C66" s="134"/>
+      <c r="D66" s="135"/>
+      <c r="E66" s="27"/>
+      <c r="F66" s="27"/>
+      <c r="G66" s="51">
+        <f>G64+G19+G28+G65</f>
+        <v>273</v>
+      </c>
+      <c r="H66" s="44"/>
       <c r="I66" s="2"/>
       <c r="J66" s="2"/>
       <c r="K66" s="2"/>
@@ -6174,17 +6318,13 @@
     </row>
     <row r="67" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A67" s="3"/>
-      <c r="B67" s="58" t="s">
-        <v>41</v>
-      </c>
-      <c r="C67" s="58">
-        <f>'List - Hide'!AC11</f>
-        <v>487</v>
-      </c>
+      <c r="B67" s="2"/>
+      <c r="C67" s="2"/>
       <c r="D67" s="2"/>
+      <c r="E67" s="2"/>
       <c r="F67" s="2"/>
       <c r="G67" s="2"/>
-      <c r="H67" s="37"/>
+      <c r="H67" s="43"/>
       <c r="I67" s="2"/>
       <c r="J67" s="2"/>
       <c r="K67" s="2"/>
@@ -6222,13 +6362,7 @@
     </row>
     <row r="68" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A68" s="3"/>
-      <c r="B68" s="58" t="s">
-        <v>42</v>
-      </c>
-      <c r="C68" s="58">
-        <f>G64</f>
-        <v>189</v>
-      </c>
+      <c r="B68" s="1"/>
       <c r="D68" s="2"/>
       <c r="F68" s="2"/>
       <c r="G68" s="2"/>
@@ -6271,11 +6405,11 @@
     <row r="69" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A69" s="3"/>
       <c r="B69" s="58" t="s">
-        <v>43</v>
-      </c>
-      <c r="C69" s="60">
-        <f>C67-C68</f>
-        <v>298</v>
+        <v>41</v>
+      </c>
+      <c r="C69" s="58">
+        <f>'List - Hide'!AC11</f>
+        <v>487</v>
       </c>
       <c r="D69" s="2"/>
       <c r="F69" s="2"/>
@@ -6318,7 +6452,13 @@
     </row>
     <row r="70" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A70" s="3"/>
-      <c r="B70" s="2"/>
+      <c r="B70" s="58" t="s">
+        <v>42</v>
+      </c>
+      <c r="C70" s="58">
+        <f>G66</f>
+        <v>273</v>
+      </c>
       <c r="D70" s="2"/>
       <c r="F70" s="2"/>
       <c r="G70" s="2"/>
@@ -6360,11 +6500,17 @@
     </row>
     <row r="71" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
-      <c r="B71" s="2"/>
+      <c r="B71" s="58" t="s">
+        <v>43</v>
+      </c>
+      <c r="C71" s="60">
+        <f>C69-C70</f>
+        <v>214</v>
+      </c>
       <c r="D71" s="2"/>
       <c r="F71" s="2"/>
       <c r="G71" s="2"/>
-      <c r="H71" s="2"/>
+      <c r="H71" s="37"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
       <c r="K71" s="2"/>
@@ -6406,7 +6552,7 @@
       <c r="D72" s="2"/>
       <c r="F72" s="2"/>
       <c r="G72" s="2"/>
-      <c r="H72" s="2"/>
+      <c r="H72" s="37"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
@@ -6445,9 +6591,7 @@
     <row r="73" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A73" s="3"/>
       <c r="B73" s="2"/>
-      <c r="C73" s="2"/>
       <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
       <c r="F73" s="2"/>
       <c r="G73" s="2"/>
       <c r="H73" s="2"/>
@@ -6489,9 +6633,7 @@
     <row r="74" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A74" s="3"/>
       <c r="B74" s="2"/>
-      <c r="C74" s="2"/>
       <c r="D74" s="2"/>
-      <c r="E74" s="2"/>
       <c r="F74" s="2"/>
       <c r="G74" s="2"/>
       <c r="H74" s="2"/>
@@ -6627,7 +6769,7 @@
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
       <c r="H77" s="2"/>
-      <c r="I77" s="4"/>
+      <c r="I77" s="2"/>
       <c r="J77" s="2"/>
       <c r="K77" s="2"/>
       <c r="L77" s="2"/>
@@ -6671,7 +6813,7 @@
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
       <c r="H78" s="2"/>
-      <c r="I78" s="5"/>
+      <c r="I78" s="2"/>
       <c r="J78" s="2"/>
       <c r="K78" s="2"/>
       <c r="L78" s="2"/>
@@ -6707,7 +6849,7 @@
       <c r="AP78" s="2"/>
     </row>
     <row r="79" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="A79" s="2"/>
+      <c r="A79" s="3"/>
       <c r="B79" s="2"/>
       <c r="C79" s="2"/>
       <c r="D79" s="2"/>
@@ -6715,7 +6857,7 @@
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
       <c r="H79" s="2"/>
-      <c r="I79" s="5"/>
+      <c r="I79" s="4"/>
       <c r="J79" s="2"/>
       <c r="K79" s="2"/>
       <c r="L79" s="2"/>
@@ -6751,7 +6893,7 @@
       <c r="AP79" s="2"/>
     </row>
     <row r="80" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="A80" s="2"/>
+      <c r="A80" s="3"/>
       <c r="B80" s="2"/>
       <c r="C80" s="2"/>
       <c r="D80" s="2"/>
@@ -6759,7 +6901,7 @@
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
       <c r="H80" s="2"/>
-      <c r="I80" s="2"/>
+      <c r="I80" s="5"/>
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
       <c r="L80" s="2"/>
@@ -6803,7 +6945,7 @@
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
       <c r="H81" s="2"/>
-      <c r="I81" s="2"/>
+      <c r="I81" s="5"/>
       <c r="J81" s="2"/>
       <c r="K81" s="2"/>
       <c r="L81" s="2"/>
@@ -7138,6 +7280,13 @@
       <c r="AG88" s="2"/>
       <c r="AH88" s="2"/>
       <c r="AI88" s="2"/>
+      <c r="AJ88" s="2"/>
+      <c r="AK88" s="2"/>
+      <c r="AL88" s="2"/>
+      <c r="AM88" s="2"/>
+      <c r="AN88" s="2"/>
+      <c r="AO88" s="2"/>
+      <c r="AP88" s="2"/>
     </row>
     <row r="89" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A89" s="2"/>
@@ -7175,6 +7324,13 @@
       <c r="AG89" s="2"/>
       <c r="AH89" s="2"/>
       <c r="AI89" s="2"/>
+      <c r="AJ89" s="2"/>
+      <c r="AK89" s="2"/>
+      <c r="AL89" s="2"/>
+      <c r="AM89" s="2"/>
+      <c r="AN89" s="2"/>
+      <c r="AO89" s="2"/>
+      <c r="AP89" s="2"/>
     </row>
     <row r="90" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A90" s="2"/>
@@ -7695,7 +7851,7 @@
       <c r="AI103" s="2"/>
     </row>
     <row r="104" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A104" s="3"/>
+      <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
       <c r="D104" s="2"/>
@@ -7732,7 +7888,7 @@
       <c r="AI104" s="2"/>
     </row>
     <row r="105" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A105" s="3"/>
+      <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="2"/>
       <c r="D105" s="2"/>
@@ -7843,6 +7999,7 @@
       <c r="AI107" s="2"/>
     </row>
     <row r="108" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A108" s="3"/>
       <c r="B108" s="2"/>
       <c r="C108" s="2"/>
       <c r="D108" s="2"/>
@@ -7879,7 +8036,7 @@
       <c r="AI108" s="2"/>
     </row>
     <row r="109" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A109" s="4"/>
+      <c r="A109" s="3"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
       <c r="D109" s="2"/>
@@ -7916,7 +8073,6 @@
       <c r="AI109" s="2"/>
     </row>
     <row r="110" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
       <c r="D110" s="2"/>
@@ -7953,7 +8109,7 @@
       <c r="AI110" s="2"/>
     </row>
     <row r="111" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A111" s="2"/>
+      <c r="A111" s="4"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
       <c r="D111" s="2"/>
@@ -9192,8 +9348,25 @@
       <c r="P144" s="2"/>
       <c r="Q144" s="2"/>
       <c r="R144" s="2"/>
-    </row>
-    <row r="145" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S144" s="2"/>
+      <c r="T144" s="2"/>
+      <c r="U144" s="2"/>
+      <c r="V144" s="2"/>
+      <c r="W144" s="2"/>
+      <c r="X144" s="2"/>
+      <c r="Y144" s="2"/>
+      <c r="Z144" s="2"/>
+      <c r="AA144" s="2"/>
+      <c r="AB144" s="2"/>
+      <c r="AC144" s="2"/>
+      <c r="AD144" s="2"/>
+      <c r="AE144" s="2"/>
+      <c r="AF144" s="2"/>
+      <c r="AG144" s="2"/>
+      <c r="AH144" s="2"/>
+      <c r="AI144" s="2"/>
+    </row>
+    <row r="145" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A145" s="2"/>
       <c r="B145" s="2"/>
       <c r="C145" s="2"/>
@@ -9212,8 +9385,25 @@
       <c r="P145" s="2"/>
       <c r="Q145" s="2"/>
       <c r="R145" s="2"/>
-    </row>
-    <row r="146" spans="1:18" x14ac:dyDescent="0.25">
+      <c r="S145" s="2"/>
+      <c r="T145" s="2"/>
+      <c r="U145" s="2"/>
+      <c r="V145" s="2"/>
+      <c r="W145" s="2"/>
+      <c r="X145" s="2"/>
+      <c r="Y145" s="2"/>
+      <c r="Z145" s="2"/>
+      <c r="AA145" s="2"/>
+      <c r="AB145" s="2"/>
+      <c r="AC145" s="2"/>
+      <c r="AD145" s="2"/>
+      <c r="AE145" s="2"/>
+      <c r="AF145" s="2"/>
+      <c r="AG145" s="2"/>
+      <c r="AH145" s="2"/>
+      <c r="AI145" s="2"/>
+    </row>
+    <row r="146" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A146" s="2"/>
       <c r="B146" s="2"/>
       <c r="C146" s="2"/>
@@ -9233,7 +9423,7 @@
       <c r="Q146" s="2"/>
       <c r="R146" s="2"/>
     </row>
-    <row r="147" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="147" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A147" s="2"/>
       <c r="B147" s="2"/>
       <c r="C147" s="2"/>
@@ -9253,7 +9443,7 @@
       <c r="Q147" s="2"/>
       <c r="R147" s="2"/>
     </row>
-    <row r="148" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="148" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A148" s="2"/>
       <c r="B148" s="2"/>
       <c r="C148" s="2"/>
@@ -9273,7 +9463,7 @@
       <c r="Q148" s="2"/>
       <c r="R148" s="2"/>
     </row>
-    <row r="149" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="149" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A149" s="2"/>
       <c r="B149" s="2"/>
       <c r="C149" s="2"/>
@@ -9293,7 +9483,7 @@
       <c r="Q149" s="2"/>
       <c r="R149" s="2"/>
     </row>
-    <row r="150" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="150" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A150" s="2"/>
       <c r="B150" s="2"/>
       <c r="C150" s="2"/>
@@ -9313,7 +9503,7 @@
       <c r="Q150" s="2"/>
       <c r="R150" s="2"/>
     </row>
-    <row r="151" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="151" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A151" s="2"/>
       <c r="B151" s="2"/>
       <c r="C151" s="2"/>
@@ -9333,7 +9523,7 @@
       <c r="Q151" s="2"/>
       <c r="R151" s="2"/>
     </row>
-    <row r="152" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="152" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A152" s="2"/>
       <c r="B152" s="2"/>
       <c r="C152" s="2"/>
@@ -9353,7 +9543,7 @@
       <c r="Q152" s="2"/>
       <c r="R152" s="2"/>
     </row>
-    <row r="153" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="153" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A153" s="2"/>
       <c r="B153" s="2"/>
       <c r="C153" s="2"/>
@@ -9373,7 +9563,7 @@
       <c r="Q153" s="2"/>
       <c r="R153" s="2"/>
     </row>
-    <row r="154" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="154" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A154" s="2"/>
       <c r="B154" s="2"/>
       <c r="C154" s="2"/>
@@ -9393,7 +9583,7 @@
       <c r="Q154" s="2"/>
       <c r="R154" s="2"/>
     </row>
-    <row r="155" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="155" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A155" s="2"/>
       <c r="B155" s="2"/>
       <c r="C155" s="2"/>
@@ -9413,7 +9603,7 @@
       <c r="Q155" s="2"/>
       <c r="R155" s="2"/>
     </row>
-    <row r="156" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="156" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A156" s="2"/>
       <c r="B156" s="2"/>
       <c r="C156" s="2"/>
@@ -9433,7 +9623,7 @@
       <c r="Q156" s="2"/>
       <c r="R156" s="2"/>
     </row>
-    <row r="157" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="157" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A157" s="2"/>
       <c r="B157" s="2"/>
       <c r="C157" s="2"/>
@@ -9453,7 +9643,7 @@
       <c r="Q157" s="2"/>
       <c r="R157" s="2"/>
     </row>
-    <row r="158" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="158" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A158" s="2"/>
       <c r="B158" s="2"/>
       <c r="C158" s="2"/>
@@ -9473,7 +9663,7 @@
       <c r="Q158" s="2"/>
       <c r="R158" s="2"/>
     </row>
-    <row r="159" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="159" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A159" s="2"/>
       <c r="B159" s="2"/>
       <c r="C159" s="2"/>
@@ -9493,7 +9683,7 @@
       <c r="Q159" s="2"/>
       <c r="R159" s="2"/>
     </row>
-    <row r="160" spans="1:18" x14ac:dyDescent="0.25">
+    <row r="160" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A160" s="2"/>
       <c r="B160" s="2"/>
       <c r="C160" s="2"/>
@@ -11725,6 +11915,13 @@
       <c r="I271" s="2"/>
       <c r="J271" s="2"/>
       <c r="K271" s="2"/>
+      <c r="L271" s="2"/>
+      <c r="M271" s="2"/>
+      <c r="N271" s="2"/>
+      <c r="O271" s="2"/>
+      <c r="P271" s="2"/>
+      <c r="Q271" s="2"/>
+      <c r="R271" s="2"/>
     </row>
     <row r="272" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A272" s="2"/>
@@ -11738,6 +11935,13 @@
       <c r="I272" s="2"/>
       <c r="J272" s="2"/>
       <c r="K272" s="2"/>
+      <c r="L272" s="2"/>
+      <c r="M272" s="2"/>
+      <c r="N272" s="2"/>
+      <c r="O272" s="2"/>
+      <c r="P272" s="2"/>
+      <c r="Q272" s="2"/>
+      <c r="R272" s="2"/>
     </row>
     <row r="273" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A273" s="2"/>
@@ -12053,6 +12257,12 @@
     </row>
     <row r="297" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A297" s="2"/>
+      <c r="B297" s="2"/>
+      <c r="C297" s="2"/>
+      <c r="D297" s="2"/>
+      <c r="E297" s="2"/>
+      <c r="F297" s="2"/>
+      <c r="G297" s="2"/>
       <c r="H297" s="2"/>
       <c r="I297" s="2"/>
       <c r="J297" s="2"/>
@@ -12060,6 +12270,12 @@
     </row>
     <row r="298" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A298" s="2"/>
+      <c r="B298" s="2"/>
+      <c r="C298" s="2"/>
+      <c r="D298" s="2"/>
+      <c r="E298" s="2"/>
+      <c r="F298" s="2"/>
+      <c r="G298" s="2"/>
       <c r="H298" s="2"/>
       <c r="I298" s="2"/>
       <c r="J298" s="2"/>
@@ -12074,12 +12290,14 @@
     </row>
     <row r="300" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A300" s="2"/>
+      <c r="H300" s="2"/>
       <c r="I300" s="2"/>
       <c r="J300" s="2"/>
       <c r="K300" s="2"/>
     </row>
     <row r="301" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A301" s="2"/>
+      <c r="H301" s="2"/>
       <c r="I301" s="2"/>
       <c r="J301" s="2"/>
       <c r="K301" s="2"/>
@@ -12156,23 +12374,38 @@
       <c r="J313" s="2"/>
       <c r="K313" s="2"/>
     </row>
+    <row r="314" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A314" s="2"/>
+      <c r="I314" s="2"/>
+      <c r="J314" s="2"/>
+      <c r="K314" s="2"/>
+    </row>
+    <row r="315" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A315" s="2"/>
+      <c r="I315" s="2"/>
+      <c r="J315" s="2"/>
+      <c r="K315" s="2"/>
+    </row>
   </sheetData>
-  <mergeCells count="43">
-    <mergeCell ref="B3:G3"/>
-    <mergeCell ref="J35:O35"/>
-    <mergeCell ref="J37:O37"/>
-    <mergeCell ref="J40:O40"/>
-    <mergeCell ref="J30:O30"/>
-    <mergeCell ref="B29:H29"/>
-    <mergeCell ref="B31:F31"/>
-    <mergeCell ref="H5:H19"/>
-    <mergeCell ref="J2:O2"/>
-    <mergeCell ref="J29:O29"/>
-    <mergeCell ref="J17:O17"/>
-    <mergeCell ref="J5:O5"/>
-    <mergeCell ref="J22:O22"/>
-    <mergeCell ref="E56:F56"/>
-    <mergeCell ref="E57:F57"/>
+  <mergeCells count="45">
+    <mergeCell ref="E60:F60"/>
+    <mergeCell ref="H22:H28"/>
+    <mergeCell ref="H35:H64"/>
+    <mergeCell ref="E40:F40"/>
+    <mergeCell ref="E41:F41"/>
+    <mergeCell ref="E42:F42"/>
+    <mergeCell ref="E43:F43"/>
+    <mergeCell ref="E62:F62"/>
+    <mergeCell ref="E63:F63"/>
+    <mergeCell ref="E64:F64"/>
+    <mergeCell ref="E44:F44"/>
+    <mergeCell ref="E45:F45"/>
+    <mergeCell ref="E61:F61"/>
+    <mergeCell ref="E48:F48"/>
+    <mergeCell ref="E49:F49"/>
+    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="E58:F58"/>
+    <mergeCell ref="E59:F59"/>
     <mergeCell ref="E46:F46"/>
     <mergeCell ref="E47:F47"/>
     <mergeCell ref="E35:F35"/>
@@ -12182,25 +12415,24 @@
     <mergeCell ref="E51:F51"/>
     <mergeCell ref="E52:F52"/>
     <mergeCell ref="E53:F53"/>
+    <mergeCell ref="E56:F56"/>
+    <mergeCell ref="E57:F57"/>
+    <mergeCell ref="E38:F38"/>
     <mergeCell ref="E54:F54"/>
     <mergeCell ref="E55:F55"/>
-    <mergeCell ref="E38:F38"/>
-    <mergeCell ref="E58:F58"/>
-    <mergeCell ref="H22:H28"/>
-    <mergeCell ref="H35:H62"/>
-    <mergeCell ref="E40:F40"/>
-    <mergeCell ref="E41:F41"/>
-    <mergeCell ref="E42:F42"/>
-    <mergeCell ref="E43:F43"/>
-    <mergeCell ref="E60:F60"/>
-    <mergeCell ref="E61:F61"/>
-    <mergeCell ref="E62:F62"/>
-    <mergeCell ref="E44:F44"/>
-    <mergeCell ref="E45:F45"/>
-    <mergeCell ref="E59:F59"/>
-    <mergeCell ref="E48:F48"/>
-    <mergeCell ref="E49:F49"/>
-    <mergeCell ref="E50:F50"/>
+    <mergeCell ref="J2:O2"/>
+    <mergeCell ref="J29:O29"/>
+    <mergeCell ref="J17:O17"/>
+    <mergeCell ref="J5:O5"/>
+    <mergeCell ref="J22:O22"/>
+    <mergeCell ref="B3:G3"/>
+    <mergeCell ref="J35:O35"/>
+    <mergeCell ref="J37:O37"/>
+    <mergeCell ref="J40:O40"/>
+    <mergeCell ref="J30:O30"/>
+    <mergeCell ref="B29:H29"/>
+    <mergeCell ref="B31:F31"/>
+    <mergeCell ref="H5:H19"/>
   </mergeCells>
   <phoneticPr fontId="24" type="noConversion"/>
   <dataValidations count="6">
@@ -12226,13 +12458,13 @@
           <x14:formula1>
             <xm:f>'List - Hide'!$C$2:$C$19</xm:f>
           </x14:formula1>
-          <xm:sqref>C36:C61</xm:sqref>
+          <xm:sqref>C36:C63</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry!" error="Please pick from the list!" prompt="Please select from the list" xr:uid="{00000000-0002-0000-0000-000006000000}">
           <x14:formula1>
             <xm:f>'List - Hide'!$A$2:$A$17</xm:f>
           </x14:formula1>
-          <xm:sqref>C62:C63 C73:C91 C65</xm:sqref>
+          <xm:sqref>C64:C65 C75:C93 C67</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -12434,7 +12666,7 @@
       </c>
     </row>
     <row r="2" spans="1:53" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="86" t="s">
+      <c r="A2" s="147" t="s">
         <v>67</v>
       </c>
       <c r="B2" s="88" t="s">
@@ -12495,7 +12727,7 @@
       <c r="BA2" s="43"/>
     </row>
     <row r="3" spans="1:53" ht="60" x14ac:dyDescent="0.25">
-      <c r="A3" s="86" t="s">
+      <c r="A3" s="147" t="s">
         <v>70</v>
       </c>
       <c r="B3" s="87" t="s">
@@ -12739,13 +12971,13 @@
       <c r="BA6" s="43"/>
     </row>
     <row r="7" spans="1:53" ht="30" x14ac:dyDescent="0.25">
-      <c r="A7" s="86" t="s">
+      <c r="A7" s="147" t="s">
         <v>82</v>
       </c>
       <c r="B7" s="87" t="s">
         <v>83</v>
       </c>
-      <c r="C7" s="87" t="s">
+      <c r="C7" s="148" t="s">
         <v>84</v>
       </c>
       <c r="D7" s="43"/>
@@ -12859,7 +13091,7 @@
       <c r="BA8" s="43"/>
     </row>
     <row r="9" spans="1:53" x14ac:dyDescent="0.25">
-      <c r="A9" s="86" t="s">
+      <c r="A9" s="147" t="s">
         <v>87</v>
       </c>
       <c r="B9" s="87" t="s">
@@ -12918,7 +13150,7 @@
       <c r="BA9" s="43"/>
     </row>
     <row r="10" spans="1:53" ht="30" x14ac:dyDescent="0.25">
-      <c r="A10" s="86" t="s">
+      <c r="A10" s="147" t="s">
         <v>89</v>
       </c>
       <c r="B10" s="148" t="s">
@@ -12977,7 +13209,7 @@
       <c r="BA10" s="43"/>
     </row>
     <row r="11" spans="1:53" ht="30" x14ac:dyDescent="0.25">
-      <c r="A11" s="86" t="s">
+      <c r="A11" s="147" t="s">
         <v>91</v>
       </c>
       <c r="B11" s="87" t="s">
@@ -13390,7 +13622,7 @@
       <c r="BA17" s="43"/>
     </row>
     <row r="18" spans="1:53" ht="30" x14ac:dyDescent="0.25">
-      <c r="A18" s="86" t="s">
+      <c r="A18" s="147" t="s">
         <v>105</v>
       </c>
       <c r="B18" s="43" t="s">
@@ -13449,7 +13681,7 @@
       <c r="BA18" s="43"/>
     </row>
     <row r="19" spans="1:53" ht="30" x14ac:dyDescent="0.25">
-      <c r="A19" s="86" t="s">
+      <c r="A19" s="147" t="s">
         <v>107</v>
       </c>
       <c r="B19" s="43" t="s">
@@ -13567,7 +13799,7 @@
       <c r="BA20" s="43"/>
     </row>
     <row r="21" spans="1:53" x14ac:dyDescent="0.25">
-      <c r="A21" s="86" t="s">
+      <c r="A21" s="147" t="s">
         <v>111</v>
       </c>
       <c r="B21" s="43" t="s">
@@ -13862,7 +14094,7 @@
       <c r="BA25" s="43"/>
     </row>
     <row r="26" spans="1:53" ht="30" x14ac:dyDescent="0.25">
-      <c r="A26" s="86" t="s">
+      <c r="A26" s="147" t="s">
         <v>121</v>
       </c>
       <c r="B26" s="43" t="s">
@@ -13921,7 +14153,7 @@
       <c r="BA26" s="43"/>
     </row>
     <row r="27" spans="1:53" x14ac:dyDescent="0.25">
-      <c r="A27" s="86" t="s">
+      <c r="A27" s="147" t="s">
         <v>123</v>
       </c>
       <c r="B27" s="150" t="s">
@@ -14098,10 +14330,10 @@
       <c r="BA29" s="43"/>
     </row>
     <row r="30" spans="1:53" s="86" customFormat="1" ht="30" x14ac:dyDescent="0.25">
-      <c r="A30" s="86" t="s">
+      <c r="A30" s="147" t="s">
         <v>129</v>
       </c>
-      <c r="B30" s="87" t="s">
+      <c r="B30" s="148" t="s">
         <v>130</v>
       </c>
       <c r="C30" s="87"/>
@@ -14157,7 +14389,7 @@
       <c r="BA30" s="87"/>
     </row>
     <row r="31" spans="1:53" ht="30" x14ac:dyDescent="0.25">
-      <c r="A31" s="86" t="s">
+      <c r="A31" s="147" t="s">
         <v>131</v>
       </c>
       <c r="B31" s="43"/>
@@ -25889,10 +26121,10 @@
       <c r="AH1" s="68"/>
     </row>
     <row r="2" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="191" t="s">
+      <c r="A2" s="197" t="s">
         <v>142</v>
       </c>
-      <c r="B2" s="195">
+      <c r="B2" s="201">
         <v>1</v>
       </c>
       <c r="C2" s="72" t="s">
@@ -25948,8 +26180,8 @@
       <c r="AH2" s="69"/>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A3" s="192"/>
-      <c r="B3" s="189"/>
+      <c r="A3" s="198"/>
+      <c r="B3" s="195"/>
       <c r="C3" s="74" t="s">
         <v>144</v>
       </c>
@@ -26000,8 +26232,8 @@
       <c r="AH3" s="69"/>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A4" s="192"/>
-      <c r="B4" s="189"/>
+      <c r="A4" s="198"/>
+      <c r="B4" s="195"/>
       <c r="C4" s="74" t="s">
         <v>145</v>
       </c>
@@ -26052,8 +26284,8 @@
       <c r="AH4" s="69"/>
     </row>
     <row r="5" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="192"/>
-      <c r="B5" s="194"/>
+      <c r="A5" s="198"/>
+      <c r="B5" s="200"/>
       <c r="C5" s="74" t="s">
         <v>146</v>
       </c>
@@ -26104,8 +26336,8 @@
       <c r="AH5" s="69"/>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A6" s="192"/>
-      <c r="B6" s="189">
+      <c r="A6" s="198"/>
+      <c r="B6" s="195">
         <v>2</v>
       </c>
       <c r="C6" s="74" t="s">
@@ -26160,8 +26392,8 @@
       <c r="AH6" s="69"/>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A7" s="192"/>
-      <c r="B7" s="189"/>
+      <c r="A7" s="198"/>
+      <c r="B7" s="195"/>
       <c r="C7" s="74" t="s">
         <v>148</v>
       </c>
@@ -26212,8 +26444,8 @@
       <c r="AH7" s="69"/>
     </row>
     <row r="8" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="192"/>
-      <c r="B8" s="189"/>
+      <c r="A8" s="198"/>
+      <c r="B8" s="195"/>
       <c r="C8" s="74" t="s">
         <v>149</v>
       </c>
@@ -26263,8 +26495,8 @@
       <c r="AH8" s="69"/>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A9" s="192"/>
-      <c r="B9" s="189"/>
+      <c r="A9" s="198"/>
+      <c r="B9" s="195"/>
       <c r="C9" s="74" t="s">
         <v>150</v>
       </c>
@@ -26319,8 +26551,8 @@
       <c r="AH9" s="69"/>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A10" s="192"/>
-      <c r="B10" s="189">
+      <c r="A10" s="198"/>
+      <c r="B10" s="195">
         <v>3</v>
       </c>
       <c r="C10" s="74" t="s">
@@ -26378,8 +26610,8 @@
       <c r="AH10" s="69"/>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A11" s="192"/>
-      <c r="B11" s="189"/>
+      <c r="A11" s="198"/>
+      <c r="B11" s="195"/>
       <c r="C11" s="74" t="s">
         <v>155</v>
       </c>
@@ -26434,8 +26666,8 @@
       <c r="AH11" s="69"/>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A12" s="192"/>
-      <c r="B12" s="189"/>
+      <c r="A12" s="198"/>
+      <c r="B12" s="195"/>
       <c r="C12" s="74" t="s">
         <v>157</v>
       </c>
@@ -26493,8 +26725,8 @@
       <c r="AH12" s="69"/>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A13" s="192"/>
-      <c r="B13" s="189"/>
+      <c r="A13" s="198"/>
+      <c r="B13" s="195"/>
       <c r="C13" s="74" t="s">
         <v>162</v>
       </c>
@@ -26560,8 +26792,8 @@
       <c r="AH13" s="69"/>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A14" s="192"/>
-      <c r="B14" s="189">
+      <c r="A14" s="198"/>
+      <c r="B14" s="195">
         <v>4</v>
       </c>
       <c r="C14" s="74" t="s">
@@ -26628,8 +26860,8 @@
       <c r="AH14" s="69"/>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A15" s="192"/>
-      <c r="B15" s="189"/>
+      <c r="A15" s="198"/>
+      <c r="B15" s="195"/>
       <c r="C15" s="74" t="s">
         <v>165</v>
       </c>
@@ -26692,8 +26924,8 @@
       <c r="AH15" s="69"/>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A16" s="192"/>
-      <c r="B16" s="189"/>
+      <c r="A16" s="198"/>
+      <c r="B16" s="195"/>
       <c r="C16" s="74" t="s">
         <v>166</v>
       </c>
@@ -26756,8 +26988,8 @@
       <c r="AH16" s="69"/>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A17" s="192"/>
-      <c r="B17" s="189"/>
+      <c r="A17" s="198"/>
+      <c r="B17" s="195"/>
       <c r="C17" s="74" t="s">
         <v>167</v>
       </c>
@@ -26820,8 +27052,8 @@
       <c r="AH17" s="69"/>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A18" s="192"/>
-      <c r="B18" s="189">
+      <c r="A18" s="198"/>
+      <c r="B18" s="195">
         <v>5</v>
       </c>
       <c r="C18" s="74" t="s">
@@ -26888,8 +27120,8 @@
       <c r="AH18" s="69"/>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A19" s="192"/>
-      <c r="B19" s="189"/>
+      <c r="A19" s="198"/>
+      <c r="B19" s="195"/>
       <c r="C19" s="74" t="s">
         <v>169</v>
       </c>
@@ -26953,8 +27185,8 @@
       <c r="AH19" s="69"/>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A20" s="192"/>
-      <c r="B20" s="189"/>
+      <c r="A20" s="198"/>
+      <c r="B20" s="195"/>
       <c r="C20" s="74" t="s">
         <v>170</v>
       </c>
@@ -27017,8 +27249,8 @@
       <c r="AH20" s="69"/>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A21" s="192"/>
-      <c r="B21" s="189"/>
+      <c r="A21" s="198"/>
+      <c r="B21" s="195"/>
       <c r="C21" s="74" t="s">
         <v>171</v>
       </c>
@@ -27081,8 +27313,8 @@
       <c r="AG21" s="85"/>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A22" s="192"/>
-      <c r="B22" s="189">
+      <c r="A22" s="198"/>
+      <c r="B22" s="195">
         <v>6</v>
       </c>
       <c r="C22" s="74" t="s">
@@ -27148,8 +27380,8 @@
       <c r="AG22" s="85"/>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A23" s="192"/>
-      <c r="B23" s="189"/>
+      <c r="A23" s="198"/>
+      <c r="B23" s="195"/>
       <c r="C23" s="74" t="s">
         <v>173</v>
       </c>
@@ -27214,8 +27446,8 @@
       <c r="AG23" s="85"/>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A24" s="192"/>
-      <c r="B24" s="189"/>
+      <c r="A24" s="198"/>
+      <c r="B24" s="195"/>
       <c r="C24" s="74" t="s">
         <v>174</v>
       </c>
@@ -27276,8 +27508,8 @@
       <c r="AG24" s="85"/>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A25" s="192"/>
-      <c r="B25" s="189"/>
+      <c r="A25" s="198"/>
+      <c r="B25" s="195"/>
       <c r="C25" s="74" t="s">
         <v>175</v>
       </c>
@@ -27335,8 +27567,8 @@
       <c r="AG25" s="69"/>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A26" s="192"/>
-      <c r="B26" s="189">
+      <c r="A26" s="198"/>
+      <c r="B26" s="195">
         <v>7</v>
       </c>
       <c r="C26" s="74" t="s">
@@ -27396,8 +27628,8 @@
       <c r="AG26" s="69"/>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A27" s="192"/>
-      <c r="B27" s="189"/>
+      <c r="A27" s="198"/>
+      <c r="B27" s="195"/>
       <c r="C27" s="74" t="s">
         <v>177</v>
       </c>
@@ -27453,8 +27685,8 @@
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A28" s="192"/>
-      <c r="B28" s="189"/>
+      <c r="A28" s="198"/>
+      <c r="B28" s="195"/>
       <c r="C28" s="74" t="s">
         <v>179</v>
       </c>
@@ -27510,8 +27742,8 @@
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A29" s="192"/>
-      <c r="B29" s="189"/>
+      <c r="A29" s="198"/>
+      <c r="B29" s="195"/>
       <c r="C29" s="74" t="s">
         <v>181</v>
       </c>
@@ -27568,8 +27800,8 @@
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A30" s="192"/>
-      <c r="B30" s="189">
+      <c r="A30" s="198"/>
+      <c r="B30" s="195">
         <v>8</v>
       </c>
       <c r="C30" s="74" t="s">
@@ -27627,8 +27859,8 @@
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A31" s="192"/>
-      <c r="B31" s="189"/>
+      <c r="A31" s="198"/>
+      <c r="B31" s="195"/>
       <c r="C31" s="74" t="s">
         <v>186</v>
       </c>
@@ -27683,8 +27915,8 @@
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A32" s="192"/>
-      <c r="B32" s="189"/>
+      <c r="A32" s="198"/>
+      <c r="B32" s="195"/>
       <c r="C32" s="74" t="s">
         <v>188</v>
       </c>
@@ -27734,8 +27966,8 @@
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A33" s="192"/>
-      <c r="B33" s="189"/>
+      <c r="A33" s="198"/>
+      <c r="B33" s="195"/>
       <c r="C33" s="74" t="s">
         <v>189</v>
       </c>
@@ -27781,8 +28013,8 @@
       <c r="AA33" s="69"/>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A34" s="192"/>
-      <c r="B34" s="189">
+      <c r="A34" s="198"/>
+      <c r="B34" s="195">
         <v>9</v>
       </c>
       <c r="C34" s="74" t="s">
@@ -27828,8 +28060,8 @@
       <c r="AA34" s="69"/>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A35" s="192"/>
-      <c r="B35" s="189"/>
+      <c r="A35" s="198"/>
+      <c r="B35" s="195"/>
       <c r="C35" s="74" t="s">
         <v>191</v>
       </c>
@@ -27872,8 +28104,8 @@
       <c r="AA35" s="69"/>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A36" s="192"/>
-      <c r="B36" s="189"/>
+      <c r="A36" s="198"/>
+      <c r="B36" s="195"/>
       <c r="C36" s="74" t="s">
         <v>192</v>
       </c>
@@ -27918,8 +28150,8 @@
       <c r="AA36" s="69"/>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A37" s="192"/>
-      <c r="B37" s="189"/>
+      <c r="A37" s="198"/>
+      <c r="B37" s="195"/>
       <c r="C37" s="74" t="s">
         <v>193</v>
       </c>
@@ -27962,8 +28194,8 @@
       <c r="AA37" s="69"/>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A38" s="192"/>
-      <c r="B38" s="189">
+      <c r="A38" s="198"/>
+      <c r="B38" s="195">
         <v>10</v>
       </c>
       <c r="C38" s="74" t="s">
@@ -28011,8 +28243,8 @@
       <c r="AH38" s="69"/>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A39" s="192"/>
-      <c r="B39" s="189"/>
+      <c r="A39" s="198"/>
+      <c r="B39" s="195"/>
       <c r="C39" s="74" t="s">
         <v>195</v>
       </c>
@@ -28057,8 +28289,8 @@
       <c r="AH39" s="69"/>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A40" s="192"/>
-      <c r="B40" s="189"/>
+      <c r="A40" s="198"/>
+      <c r="B40" s="195"/>
       <c r="C40" s="74" t="s">
         <v>196</v>
       </c>
@@ -28102,8 +28334,8 @@
       <c r="AH40" s="69"/>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A41" s="192"/>
-      <c r="B41" s="189"/>
+      <c r="A41" s="198"/>
+      <c r="B41" s="195"/>
       <c r="C41" s="74" t="s">
         <v>197</v>
       </c>
@@ -28153,8 +28385,8 @@
       <c r="AH41" s="69"/>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A42" s="192"/>
-      <c r="B42" s="189">
+      <c r="A42" s="198"/>
+      <c r="B42" s="195">
         <v>11</v>
       </c>
       <c r="C42" s="74" t="s">
@@ -28207,8 +28439,8 @@
       <c r="AH42" s="69"/>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A43" s="192"/>
-      <c r="B43" s="189"/>
+      <c r="A43" s="198"/>
+      <c r="B43" s="195"/>
       <c r="C43" s="74" t="s">
         <v>199</v>
       </c>
@@ -28261,8 +28493,8 @@
       <c r="AH43" s="69"/>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A44" s="192"/>
-      <c r="B44" s="189"/>
+      <c r="A44" s="198"/>
+      <c r="B44" s="195"/>
       <c r="C44" s="74" t="s">
         <v>200</v>
       </c>
@@ -28312,8 +28544,8 @@
       <c r="AH44" s="69"/>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A45" s="192"/>
-      <c r="B45" s="189"/>
+      <c r="A45" s="198"/>
+      <c r="B45" s="195"/>
       <c r="C45" s="74" t="s">
         <v>201</v>
       </c>
@@ -28363,8 +28595,8 @@
       <c r="AH45" s="69"/>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A46" s="192"/>
-      <c r="B46" s="189">
+      <c r="A46" s="198"/>
+      <c r="B46" s="195">
         <v>12</v>
       </c>
       <c r="C46" s="74" t="s">
@@ -28418,8 +28650,8 @@
       <c r="AH46" s="69"/>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A47" s="192"/>
-      <c r="B47" s="189"/>
+      <c r="A47" s="198"/>
+      <c r="B47" s="195"/>
       <c r="C47" s="74" t="s">
         <v>203</v>
       </c>
@@ -28469,8 +28701,8 @@
       <c r="AH47" s="69"/>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A48" s="192"/>
-      <c r="B48" s="189"/>
+      <c r="A48" s="198"/>
+      <c r="B48" s="195"/>
       <c r="C48" s="74" t="s">
         <v>204</v>
       </c>
@@ -28522,8 +28754,8 @@
       <c r="AH48" s="69"/>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A49" s="192"/>
-      <c r="B49" s="189"/>
+      <c r="A49" s="198"/>
+      <c r="B49" s="195"/>
       <c r="C49" s="74" t="s">
         <v>205</v>
       </c>
@@ -28573,8 +28805,8 @@
       <c r="AH49" s="69"/>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A50" s="192"/>
-      <c r="B50" s="189">
+      <c r="A50" s="198"/>
+      <c r="B50" s="195">
         <v>13</v>
       </c>
       <c r="C50" s="74" t="s">
@@ -28628,8 +28860,8 @@
       <c r="AH50" s="69"/>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A51" s="192"/>
-      <c r="B51" s="189"/>
+      <c r="A51" s="198"/>
+      <c r="B51" s="195"/>
       <c r="C51" s="74" t="s">
         <v>207</v>
       </c>
@@ -28679,8 +28911,8 @@
       <c r="AH51" s="69"/>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A52" s="192"/>
-      <c r="B52" s="189"/>
+      <c r="A52" s="198"/>
+      <c r="B52" s="195"/>
       <c r="C52" s="74" t="s">
         <v>208</v>
       </c>
@@ -28729,8 +28961,8 @@
       <c r="AH52" s="69"/>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A53" s="192"/>
-      <c r="B53" s="189"/>
+      <c r="A53" s="198"/>
+      <c r="B53" s="195"/>
       <c r="C53" s="74" t="s">
         <v>209</v>
       </c>
@@ -28780,8 +29012,8 @@
       <c r="AH53" s="69"/>
     </row>
     <row r="54" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="192"/>
-      <c r="B54" s="189">
+      <c r="A54" s="198"/>
+      <c r="B54" s="195">
         <v>14</v>
       </c>
       <c r="C54" s="74" t="s">
@@ -28835,8 +29067,8 @@
       <c r="AH54" s="69"/>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A55" s="192"/>
-      <c r="B55" s="189"/>
+      <c r="A55" s="198"/>
+      <c r="B55" s="195"/>
       <c r="C55" s="74" t="s">
         <v>211</v>
       </c>
@@ -28887,8 +29119,8 @@
       <c r="AH55" s="69"/>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A56" s="192"/>
-      <c r="B56" s="189"/>
+      <c r="A56" s="198"/>
+      <c r="B56" s="195"/>
       <c r="C56" s="74" t="s">
         <v>212</v>
       </c>
@@ -28938,8 +29170,8 @@
       <c r="AH56" s="69"/>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A57" s="192"/>
-      <c r="B57" s="189"/>
+      <c r="A57" s="198"/>
+      <c r="B57" s="195"/>
       <c r="C57" s="74" t="s">
         <v>213</v>
       </c>
@@ -28990,8 +29222,8 @@
       <c r="AH57" s="69"/>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A58" s="192"/>
-      <c r="B58" s="189">
+      <c r="A58" s="198"/>
+      <c r="B58" s="195">
         <v>15</v>
       </c>
       <c r="C58" s="74" t="s">
@@ -29046,8 +29278,8 @@
       <c r="AH58" s="69"/>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A59" s="192"/>
-      <c r="B59" s="189"/>
+      <c r="A59" s="198"/>
+      <c r="B59" s="195"/>
       <c r="C59" s="74" t="s">
         <v>215</v>
       </c>
@@ -29098,8 +29330,8 @@
       <c r="AH59" s="69"/>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A60" s="192"/>
-      <c r="B60" s="189"/>
+      <c r="A60" s="198"/>
+      <c r="B60" s="195"/>
       <c r="C60" s="74" t="s">
         <v>216</v>
       </c>
@@ -29150,8 +29382,8 @@
       <c r="AH60" s="69"/>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A61" s="193"/>
-      <c r="B61" s="190"/>
+      <c r="A61" s="199"/>
+      <c r="B61" s="196"/>
       <c r="C61" s="76" t="s">
         <v>217</v>
       </c>
@@ -29202,10 +29434,10 @@
       <c r="AH61" s="69"/>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A62" s="191" t="s">
+      <c r="A62" s="197" t="s">
         <v>136</v>
       </c>
-      <c r="B62" s="194">
+      <c r="B62" s="200">
         <v>16</v>
       </c>
       <c r="C62" s="74" t="s">
@@ -29257,8 +29489,8 @@
       <c r="AH62" s="69"/>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A63" s="192"/>
-      <c r="B63" s="189"/>
+      <c r="A63" s="198"/>
+      <c r="B63" s="195"/>
       <c r="C63" s="74" t="s">
         <v>219</v>
       </c>
@@ -29308,8 +29540,8 @@
       <c r="AH63" s="69"/>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A64" s="192"/>
-      <c r="B64" s="189"/>
+      <c r="A64" s="198"/>
+      <c r="B64" s="195"/>
       <c r="C64" s="74" t="s">
         <v>220</v>
       </c>
@@ -29359,8 +29591,8 @@
       <c r="AH64" s="69"/>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A65" s="192"/>
-      <c r="B65" s="189"/>
+      <c r="A65" s="198"/>
+      <c r="B65" s="195"/>
       <c r="C65" s="74" t="s">
         <v>221</v>
       </c>
@@ -29410,8 +29642,8 @@
       <c r="AH65" s="69"/>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A66" s="192"/>
-      <c r="B66" s="189">
+      <c r="A66" s="198"/>
+      <c r="B66" s="195">
         <v>17</v>
       </c>
       <c r="C66" s="74" t="s">
@@ -29463,8 +29695,8 @@
       <c r="AH66" s="69"/>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A67" s="192"/>
-      <c r="B67" s="189"/>
+      <c r="A67" s="198"/>
+      <c r="B67" s="195"/>
       <c r="C67" s="74" t="s">
         <v>223</v>
       </c>
@@ -29514,8 +29746,8 @@
       <c r="AH67" s="69"/>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A68" s="192"/>
-      <c r="B68" s="189"/>
+      <c r="A68" s="198"/>
+      <c r="B68" s="195"/>
       <c r="C68" s="74" t="s">
         <v>224</v>
       </c>
@@ -29565,8 +29797,8 @@
       <c r="AH68" s="69"/>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A69" s="192"/>
-      <c r="B69" s="189"/>
+      <c r="A69" s="198"/>
+      <c r="B69" s="195"/>
       <c r="C69" s="74" t="s">
         <v>225</v>
       </c>
@@ -29616,8 +29848,8 @@
       <c r="AH69" s="69"/>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A70" s="192"/>
-      <c r="B70" s="189">
+      <c r="A70" s="198"/>
+      <c r="B70" s="195">
         <v>18</v>
       </c>
       <c r="C70" s="74" t="s">
@@ -29669,8 +29901,8 @@
       <c r="AH70" s="69"/>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A71" s="192"/>
-      <c r="B71" s="189"/>
+      <c r="A71" s="198"/>
+      <c r="B71" s="195"/>
       <c r="C71" s="74" t="s">
         <v>227</v>
       </c>
@@ -29720,8 +29952,8 @@
       <c r="AH71" s="69"/>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A72" s="192"/>
-      <c r="B72" s="189"/>
+      <c r="A72" s="198"/>
+      <c r="B72" s="195"/>
       <c r="C72" s="74" t="s">
         <v>228</v>
       </c>
@@ -29771,8 +30003,8 @@
       <c r="AH72" s="69"/>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A73" s="192"/>
-      <c r="B73" s="189"/>
+      <c r="A73" s="198"/>
+      <c r="B73" s="195"/>
       <c r="C73" s="74" t="s">
         <v>229</v>
       </c>
@@ -29822,8 +30054,8 @@
       <c r="AH73" s="69"/>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A74" s="192"/>
-      <c r="B74" s="189">
+      <c r="A74" s="198"/>
+      <c r="B74" s="195">
         <v>19</v>
       </c>
       <c r="C74" s="74" t="s">
@@ -29875,8 +30107,8 @@
       <c r="AH74" s="69"/>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A75" s="192"/>
-      <c r="B75" s="189"/>
+      <c r="A75" s="198"/>
+      <c r="B75" s="195"/>
       <c r="C75" s="74" t="s">
         <v>231</v>
       </c>
@@ -29926,8 +30158,8 @@
       <c r="AH75" s="69"/>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A76" s="192"/>
-      <c r="B76" s="189"/>
+      <c r="A76" s="198"/>
+      <c r="B76" s="195"/>
       <c r="C76" s="74" t="s">
         <v>232</v>
       </c>
@@ -29977,8 +30209,8 @@
       <c r="AH76" s="69"/>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A77" s="193"/>
-      <c r="B77" s="190"/>
+      <c r="A77" s="199"/>
+      <c r="B77" s="196"/>
       <c r="C77" s="76" t="s">
         <v>233</v>
       </c>
@@ -30165,10 +30397,10 @@
     <row r="80" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="69"/>
       <c r="B80" s="69"/>
-      <c r="C80" s="198" t="s">
+      <c r="C80" s="191" t="s">
         <v>234</v>
       </c>
-      <c r="D80" s="199"/>
+      <c r="D80" s="192"/>
       <c r="E80" s="73">
         <v>60</v>
       </c>
@@ -30207,10 +30439,10 @@
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A81" s="69"/>
       <c r="B81" s="69"/>
-      <c r="C81" s="200" t="s">
+      <c r="C81" s="193" t="s">
         <v>236</v>
       </c>
-      <c r="D81" s="201"/>
+      <c r="D81" s="194"/>
       <c r="E81" s="75">
         <v>322.5</v>
       </c>
@@ -30247,10 +30479,10 @@
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A82" s="69"/>
       <c r="B82" s="69"/>
-      <c r="C82" s="200" t="s">
+      <c r="C82" s="193" t="s">
         <v>237</v>
       </c>
-      <c r="D82" s="201"/>
+      <c r="D82" s="194"/>
       <c r="E82" s="75">
         <v>35</v>
       </c>
@@ -30287,10 +30519,10 @@
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A83" s="69"/>
       <c r="B83" s="69"/>
-      <c r="C83" s="200" t="s">
+      <c r="C83" s="193" t="s">
         <v>238</v>
       </c>
-      <c r="D83" s="201"/>
+      <c r="D83" s="194"/>
       <c r="E83" s="75">
         <v>287</v>
       </c>
@@ -30327,10 +30559,10 @@
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A84" s="69"/>
       <c r="B84" s="69"/>
-      <c r="C84" s="200" t="s">
+      <c r="C84" s="193" t="s">
         <v>239</v>
       </c>
-      <c r="D84" s="201"/>
+      <c r="D84" s="194"/>
       <c r="E84" s="75">
         <v>60</v>
       </c>
@@ -30367,10 +30599,10 @@
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A85" s="69"/>
       <c r="B85" s="69"/>
-      <c r="C85" s="196" t="s">
+      <c r="C85" s="189" t="s">
         <v>240</v>
       </c>
-      <c r="D85" s="197"/>
+      <c r="D85" s="190"/>
       <c r="E85" s="77">
         <f>Y79</f>
         <v>483</v>
@@ -30438,17 +30670,6 @@
     </row>
   </sheetData>
   <mergeCells count="27">
-    <mergeCell ref="C85:D85"/>
-    <mergeCell ref="C80:D80"/>
-    <mergeCell ref="C81:D81"/>
-    <mergeCell ref="C82:D82"/>
-    <mergeCell ref="C83:D83"/>
-    <mergeCell ref="C84:D84"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="B38:B41"/>
     <mergeCell ref="B66:B69"/>
     <mergeCell ref="B70:B73"/>
     <mergeCell ref="B74:B77"/>
@@ -30465,6 +30686,17 @@
     <mergeCell ref="B42:B45"/>
     <mergeCell ref="B46:B49"/>
     <mergeCell ref="B50:B53"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="B38:B41"/>
+    <mergeCell ref="C85:D85"/>
+    <mergeCell ref="C80:D80"/>
+    <mergeCell ref="C81:D81"/>
+    <mergeCell ref="C82:D82"/>
+    <mergeCell ref="C83:D83"/>
+    <mergeCell ref="C84:D84"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -30826,25 +31058,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="d03ffd70-462c-4172-9015-a0cdff42c83c">
-      <UserInfo>
-        <DisplayName>Craig Stevens</DisplayName>
-        <AccountId>17</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Afzan Matloob</DisplayName>
-        <AccountId>46</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65f98c99-c090-489b-8346-b847c18a5011">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -31065,21 +31284,31 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="d03ffd70-462c-4172-9015-a0cdff42c83c">
+      <UserInfo>
+        <DisplayName>Craig Stevens</DisplayName>
+        <AccountId>17</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Afzan Matloob</DisplayName>
+        <AccountId>46</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65f98c99-c090-489b-8346-b847c18a5011">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F627C2A1-639E-4000-94D7-FA9740411AFB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7D0D882-CBE1-41A5-A59C-C48B26872275}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d03ffd70-462c-4172-9015-a0cdff42c83c"/>
-    <ds:schemaRef ds:uri="65f98c99-c090-489b-8346-b847c18a5011"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -31104,9 +31333,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7D0D882-CBE1-41A5-A59C-C48B26872275}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F627C2A1-639E-4000-94D7-FA9740411AFB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d03ffd70-462c-4172-9015-a0cdff42c83c"/>
+    <ds:schemaRef ds:uri="65f98c99-c090-489b-8346-b847c18a5011"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>

<commit_message>
Update OTJ tracker - April
</commit_message>
<xml_diff>
--- a/Halyna Maslak OTJ Tracker DE L5.xlsx
+++ b/Halyna Maslak OTJ Tracker DE L5.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\DE Apprenticeship\Learning-Journal\Learning-Journal\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C1B38693-8D1E-4A5A-8FE1-2D0BA0BC579A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE2B5DCD-EAF1-4F30-8917-DDBE5A350D16}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="399" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="407" uniqueCount="325">
   <si>
     <t xml:space="preserve">Apprenticeship Training Log </t>
   </si>
@@ -1060,6 +1060,21 @@
   </si>
   <si>
     <t>S18</t>
+  </si>
+  <si>
+    <t>Harness CI pipeline</t>
+  </si>
+  <si>
+    <t>Power Automate flows</t>
+  </si>
+  <si>
+    <t>Data Quality Controls</t>
+  </si>
+  <si>
+    <t>S3</t>
+  </si>
+  <si>
+    <t>Data Product Design</t>
   </si>
 </sst>
 </file>
@@ -2390,125 +2405,8 @@
     <xf numFmtId="0" fontId="22" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -2543,12 +2441,6 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="25" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="58" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
     </xf>
@@ -2557,9 +2449,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="60" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
@@ -2587,6 +2476,132 @@
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="18" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="6" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="4" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="5" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="11" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="26" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="23" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="36" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="32" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="39" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" textRotation="90" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="37" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="35" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="30" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="33" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="31" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="0" borderId="34" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -3002,7 +3017,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:AP321"/>
+  <dimension ref="A1:AP325"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="11.7109375" customWidth="1"/>
@@ -3065,12 +3080,12 @@
       <c r="G2" s="2"/>
       <c r="H2" s="2"/>
       <c r="I2" s="2"/>
-      <c r="J2" s="157"/>
-      <c r="K2" s="158"/>
-      <c r="L2" s="158"/>
-      <c r="M2" s="158"/>
-      <c r="N2" s="158"/>
-      <c r="O2" s="159"/>
+      <c r="J2" s="171"/>
+      <c r="K2" s="172"/>
+      <c r="L2" s="172"/>
+      <c r="M2" s="172"/>
+      <c r="N2" s="172"/>
+      <c r="O2" s="173"/>
       <c r="P2" s="35"/>
       <c r="Q2" s="35"/>
       <c r="R2" s="2"/>
@@ -3101,14 +3116,14 @@
     </row>
     <row r="3" spans="1:42" ht="220.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A3" s="6"/>
-      <c r="B3" s="143" t="s">
+      <c r="B3" s="177" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="143"/>
-      <c r="D3" s="143"/>
-      <c r="E3" s="143"/>
-      <c r="F3" s="143"/>
-      <c r="G3" s="144"/>
+      <c r="C3" s="177"/>
+      <c r="D3" s="177"/>
+      <c r="E3" s="177"/>
+      <c r="F3" s="177"/>
+      <c r="G3" s="178"/>
       <c r="H3" s="1"/>
       <c r="I3" s="2"/>
       <c r="J3" s="51"/>
@@ -3206,14 +3221,14 @@
       <c r="G5" s="54" t="s">
         <v>7</v>
       </c>
-      <c r="H5" s="178"/>
+      <c r="H5" s="191"/>
       <c r="I5" s="2"/>
-      <c r="J5" s="145"/>
-      <c r="K5" s="146"/>
-      <c r="L5" s="146"/>
-      <c r="M5" s="146"/>
-      <c r="N5" s="146"/>
-      <c r="O5" s="147"/>
+      <c r="J5" s="174"/>
+      <c r="K5" s="175"/>
+      <c r="L5" s="175"/>
+      <c r="M5" s="175"/>
+      <c r="N5" s="175"/>
+      <c r="O5" s="176"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
       <c r="R5" s="2"/>
@@ -3261,7 +3276,7 @@
         <f t="shared" ref="G6:G18" si="0">IF(NOT(ISBLANK(D6)), SUM(E6:F6), 0)</f>
         <v>6</v>
       </c>
-      <c r="H6" s="178"/>
+      <c r="H6" s="191"/>
       <c r="I6" s="2"/>
       <c r="J6" s="128"/>
       <c r="K6" s="128"/>
@@ -3316,7 +3331,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="H7" s="178"/>
+      <c r="H7" s="191"/>
       <c r="I7" s="4"/>
       <c r="J7" s="2"/>
       <c r="K7" s="2"/>
@@ -3371,7 +3386,7 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="H8" s="178"/>
+      <c r="H8" s="191"/>
       <c r="I8" s="4"/>
       <c r="J8" s="3"/>
       <c r="K8" s="3"/>
@@ -3426,7 +3441,7 @@
         <f t="shared" si="0"/>
         <v>54</v>
       </c>
-      <c r="H9" s="178"/>
+      <c r="H9" s="191"/>
       <c r="I9" s="4"/>
       <c r="J9" s="3"/>
       <c r="K9" s="3"/>
@@ -3481,7 +3496,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="H10" s="178"/>
+      <c r="H10" s="191"/>
       <c r="I10" s="4"/>
       <c r="J10" s="3"/>
       <c r="K10" s="3"/>
@@ -3536,7 +3551,7 @@
         <f t="shared" si="0"/>
         <v>46</v>
       </c>
-      <c r="H11" s="178"/>
+      <c r="H11" s="191"/>
       <c r="I11" s="4"/>
       <c r="J11" s="3"/>
       <c r="K11" s="3"/>
@@ -3591,7 +3606,7 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="H12" s="178"/>
+      <c r="H12" s="191"/>
       <c r="I12" s="4"/>
       <c r="J12" s="3"/>
       <c r="K12" s="3"/>
@@ -3646,7 +3661,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="H13" s="178"/>
+      <c r="H13" s="191"/>
       <c r="I13" s="4"/>
       <c r="J13" s="3"/>
       <c r="K13" s="3"/>
@@ -3701,7 +3716,7 @@
         <f t="shared" si="0"/>
         <v>43</v>
       </c>
-      <c r="H14" s="178"/>
+      <c r="H14" s="191"/>
       <c r="I14" s="4"/>
       <c r="J14" s="3"/>
       <c r="K14" s="3"/>
@@ -3744,7 +3759,7 @@
       </c>
       <c r="C15" s="55"/>
       <c r="D15" s="76">
-        <v>45671</v>
+        <v>46036</v>
       </c>
       <c r="E15" s="55">
         <v>18</v>
@@ -3756,7 +3771,7 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="H15" s="178"/>
+      <c r="H15" s="191"/>
       <c r="I15" s="4"/>
       <c r="J15" s="3"/>
       <c r="K15" s="3"/>
@@ -3798,7 +3813,9 @@
         <v>18</v>
       </c>
       <c r="C16" s="55"/>
-      <c r="D16" s="55"/>
+      <c r="D16" s="76">
+        <v>46071</v>
+      </c>
       <c r="E16" s="55">
         <v>15</v>
       </c>
@@ -3807,9 +3824,9 @@
       </c>
       <c r="G16" s="123">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H16" s="178"/>
+        <v>27</v>
+      </c>
+      <c r="H16" s="191"/>
       <c r="I16" s="4"/>
       <c r="J16" s="3"/>
       <c r="K16" s="3"/>
@@ -3851,7 +3868,9 @@
         <v>19</v>
       </c>
       <c r="C17" s="55"/>
-      <c r="D17" s="55"/>
+      <c r="D17" s="76">
+        <v>46106</v>
+      </c>
       <c r="E17" s="55">
         <v>15</v>
       </c>
@@ -3860,16 +3879,16 @@
       </c>
       <c r="G17" s="123">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H17" s="178"/>
+        <v>27</v>
+      </c>
+      <c r="H17" s="191"/>
       <c r="I17" s="4"/>
-      <c r="J17" s="145"/>
-      <c r="K17" s="146"/>
-      <c r="L17" s="146"/>
-      <c r="M17" s="146"/>
-      <c r="N17" s="146"/>
-      <c r="O17" s="147"/>
+      <c r="J17" s="174"/>
+      <c r="K17" s="175"/>
+      <c r="L17" s="175"/>
+      <c r="M17" s="175"/>
+      <c r="N17" s="175"/>
+      <c r="O17" s="176"/>
       <c r="P17" s="2"/>
       <c r="Q17" s="2"/>
       <c r="R17" s="2"/>
@@ -3904,7 +3923,9 @@
         <v>20</v>
       </c>
       <c r="C18" s="55"/>
-      <c r="D18" s="55"/>
+      <c r="D18" s="76">
+        <v>46127</v>
+      </c>
       <c r="E18" s="55">
         <v>11</v>
       </c>
@@ -3913,9 +3934,9 @@
       </c>
       <c r="G18" s="123">
         <f t="shared" si="0"/>
-        <v>0</v>
-      </c>
-      <c r="H18" s="178"/>
+        <v>11</v>
+      </c>
+      <c r="H18" s="191"/>
       <c r="I18" s="4"/>
       <c r="J18" s="2"/>
       <c r="K18" s="2"/>
@@ -3968,9 +3989,9 @@
       </c>
       <c r="G19" s="127">
         <f>SUM(G6:G18)</f>
-        <v>304</v>
-      </c>
-      <c r="H19" s="178"/>
+        <v>369</v>
+      </c>
+      <c r="H19" s="191"/>
       <c r="I19" s="4"/>
       <c r="J19" s="2"/>
       <c r="K19" s="2"/>
@@ -4122,14 +4143,14 @@
         <f>IF(NOT(ISBLANK(D22)), SUM(E22:F22), 0)</f>
         <v>24</v>
       </c>
-      <c r="H22" s="182"/>
+      <c r="H22" s="167"/>
       <c r="I22" s="2"/>
-      <c r="J22" s="145"/>
-      <c r="K22" s="146"/>
-      <c r="L22" s="146"/>
-      <c r="M22" s="146"/>
-      <c r="N22" s="146"/>
-      <c r="O22" s="147"/>
+      <c r="J22" s="174"/>
+      <c r="K22" s="175"/>
+      <c r="L22" s="175"/>
+      <c r="M22" s="175"/>
+      <c r="N22" s="175"/>
+      <c r="O22" s="176"/>
       <c r="P22" s="2"/>
       <c r="Q22" s="2"/>
       <c r="R22" s="2"/>
@@ -4175,7 +4196,7 @@
         <f>IF(NOT(ISBLANK(D23)), SUM(E23:F23), 0)</f>
         <v>24</v>
       </c>
-      <c r="H23" s="182"/>
+      <c r="H23" s="167"/>
       <c r="I23" s="2"/>
       <c r="J23" s="2"/>
       <c r="K23" s="2"/>
@@ -4217,16 +4238,18 @@
         <v>29</v>
       </c>
       <c r="C24" s="55"/>
-      <c r="D24" s="55"/>
+      <c r="D24" s="76">
+        <v>45945</v>
+      </c>
       <c r="E24" s="55">
         <v>24</v>
       </c>
       <c r="F24" s="55"/>
       <c r="G24" s="55">
         <f>IF(NOT(ISBLANK(D24)), SUM(E24:F24), 0)</f>
-        <v>0</v>
-      </c>
-      <c r="H24" s="182"/>
+        <v>24</v>
+      </c>
+      <c r="H24" s="167"/>
       <c r="I24" s="2"/>
       <c r="J24" s="2"/>
       <c r="K24" s="2"/>
@@ -4268,16 +4291,18 @@
         <v>30</v>
       </c>
       <c r="C25" s="55"/>
-      <c r="D25" s="55"/>
+      <c r="D25" s="76">
+        <v>46063</v>
+      </c>
       <c r="E25" s="55">
         <v>24</v>
       </c>
       <c r="F25" s="55"/>
       <c r="G25" s="55">
         <f>IF(NOT(ISBLANK(D25)), SUM(E25:F25), 0)</f>
-        <v>0</v>
-      </c>
-      <c r="H25" s="182"/>
+        <v>24</v>
+      </c>
+      <c r="H25" s="167"/>
       <c r="I25" s="2"/>
       <c r="J25" s="2"/>
       <c r="K25" s="2"/>
@@ -4319,16 +4344,18 @@
         <v>31</v>
       </c>
       <c r="C26" s="55"/>
-      <c r="D26" s="55"/>
+      <c r="D26" s="76">
+        <v>46131</v>
+      </c>
       <c r="E26" s="55">
         <v>24</v>
       </c>
       <c r="F26" s="55"/>
       <c r="G26" s="55">
         <f>IF(NOT(ISBLANK(D26)), SUM(E26:F26), 0)</f>
-        <v>0</v>
-      </c>
-      <c r="H26" s="182"/>
+        <v>24</v>
+      </c>
+      <c r="H26" s="167"/>
       <c r="I26" s="2"/>
       <c r="J26" s="2"/>
       <c r="K26" s="2"/>
@@ -4372,7 +4399,7 @@
       <c r="E27" s="55"/>
       <c r="F27" s="55"/>
       <c r="G27" s="55"/>
-      <c r="H27" s="182"/>
+      <c r="H27" s="167"/>
       <c r="I27" s="2"/>
       <c r="J27" s="2"/>
       <c r="K27" s="2"/>
@@ -4425,9 +4452,9 @@
       </c>
       <c r="G28" s="57">
         <f>SUM(G22:H27)</f>
-        <v>48</v>
-      </c>
-      <c r="H28" s="182"/>
+        <v>120</v>
+      </c>
+      <c r="H28" s="167"/>
       <c r="I28" s="4"/>
       <c r="J28" s="2"/>
       <c r="K28" s="2"/>
@@ -4465,20 +4492,20 @@
     </row>
     <row r="29" spans="1:42" ht="25.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="2"/>
-      <c r="B29" s="180"/>
-      <c r="C29" s="181"/>
-      <c r="D29" s="181"/>
-      <c r="E29" s="181"/>
-      <c r="F29" s="181"/>
-      <c r="G29" s="181"/>
-      <c r="H29" s="154"/>
+      <c r="B29" s="185"/>
+      <c r="C29" s="186"/>
+      <c r="D29" s="186"/>
+      <c r="E29" s="186"/>
+      <c r="F29" s="186"/>
+      <c r="G29" s="186"/>
+      <c r="H29" s="187"/>
       <c r="I29" s="2"/>
-      <c r="J29" s="145"/>
-      <c r="K29" s="146"/>
-      <c r="L29" s="146"/>
-      <c r="M29" s="146"/>
-      <c r="N29" s="146"/>
-      <c r="O29" s="147"/>
+      <c r="J29" s="174"/>
+      <c r="K29" s="175"/>
+      <c r="L29" s="175"/>
+      <c r="M29" s="175"/>
+      <c r="N29" s="175"/>
+      <c r="O29" s="176"/>
       <c r="P29" s="2"/>
       <c r="Q29" s="2"/>
       <c r="R29" s="2"/>
@@ -4516,12 +4543,12 @@
       <c r="G30" s="2"/>
       <c r="H30" s="2"/>
       <c r="I30" s="2"/>
-      <c r="J30" s="151"/>
-      <c r="K30" s="152"/>
-      <c r="L30" s="152"/>
-      <c r="M30" s="152"/>
-      <c r="N30" s="152"/>
-      <c r="O30" s="153"/>
+      <c r="J30" s="182"/>
+      <c r="K30" s="183"/>
+      <c r="L30" s="183"/>
+      <c r="M30" s="183"/>
+      <c r="N30" s="183"/>
+      <c r="O30" s="184"/>
       <c r="P30" s="2"/>
       <c r="Q30" s="2"/>
       <c r="R30" s="2"/>
@@ -4552,13 +4579,13 @@
     </row>
     <row r="31" spans="1:42" ht="28.5" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="2"/>
-      <c r="B31" s="155" t="s">
+      <c r="B31" s="188" t="s">
         <v>33</v>
       </c>
-      <c r="C31" s="179"/>
-      <c r="D31" s="179"/>
-      <c r="E31" s="179"/>
-      <c r="F31" s="156"/>
+      <c r="C31" s="189"/>
+      <c r="D31" s="189"/>
+      <c r="E31" s="189"/>
+      <c r="F31" s="190"/>
       <c r="G31" s="2"/>
       <c r="H31" s="2"/>
       <c r="I31" s="2"/>
@@ -4741,19 +4768,19 @@
       <c r="E35" s="60" t="s">
         <v>38</v>
       </c>
-      <c r="F35" s="183" t="s">
+      <c r="F35" s="144" t="s">
         <v>25</v>
       </c>
       <c r="G35" s="139" t="s">
         <v>39</v>
       </c>
       <c r="H35" s="4"/>
-      <c r="I35" s="145"/>
-      <c r="J35" s="146"/>
-      <c r="K35" s="146"/>
-      <c r="L35" s="146"/>
-      <c r="M35" s="146"/>
-      <c r="N35" s="147"/>
+      <c r="I35" s="174"/>
+      <c r="J35" s="175"/>
+      <c r="K35" s="175"/>
+      <c r="L35" s="175"/>
+      <c r="M35" s="175"/>
+      <c r="N35" s="176"/>
       <c r="O35" s="2"/>
       <c r="P35" s="2"/>
       <c r="Q35" s="2"/>
@@ -4787,16 +4814,16 @@
       <c r="B36" s="77" t="s">
         <v>262</v>
       </c>
-      <c r="C36" s="185" t="s">
+      <c r="C36" s="146" t="s">
         <v>144</v>
       </c>
-      <c r="D36" s="186">
+      <c r="D36" s="147">
         <v>45694</v>
       </c>
-      <c r="E36" s="184" t="s">
+      <c r="E36" s="145" t="s">
         <v>263</v>
       </c>
-      <c r="F36" s="187">
+      <c r="F36" s="148">
         <v>0.5</v>
       </c>
       <c r="G36" s="140"/>
@@ -4840,26 +4867,26 @@
       <c r="B37" s="77" t="s">
         <v>264</v>
       </c>
-      <c r="C37" s="185" t="s">
+      <c r="C37" s="146" t="s">
         <v>144</v>
       </c>
-      <c r="D37" s="188">
+      <c r="D37" s="149">
         <v>45699</v>
       </c>
-      <c r="E37" s="184" t="s">
+      <c r="E37" s="145" t="s">
         <v>263</v>
       </c>
-      <c r="F37" s="187">
+      <c r="F37" s="148">
         <v>2</v>
       </c>
       <c r="G37" s="140"/>
       <c r="H37" s="5"/>
-      <c r="I37" s="148"/>
-      <c r="J37" s="149"/>
-      <c r="K37" s="149"/>
-      <c r="L37" s="149"/>
-      <c r="M37" s="149"/>
-      <c r="N37" s="150"/>
+      <c r="I37" s="179"/>
+      <c r="J37" s="180"/>
+      <c r="K37" s="180"/>
+      <c r="L37" s="180"/>
+      <c r="M37" s="180"/>
+      <c r="N37" s="181"/>
       <c r="O37" s="2"/>
       <c r="P37" s="2"/>
       <c r="Q37" s="2"/>
@@ -4893,16 +4920,16 @@
       <c r="B38" s="77" t="s">
         <v>279</v>
       </c>
-      <c r="C38" s="185" t="s">
+      <c r="C38" s="146" t="s">
         <v>143</v>
       </c>
-      <c r="D38" s="188">
+      <c r="D38" s="149">
         <v>45701</v>
       </c>
-      <c r="E38" s="184" t="s">
+      <c r="E38" s="145" t="s">
         <v>280</v>
       </c>
-      <c r="F38" s="187">
+      <c r="F38" s="148">
         <v>7</v>
       </c>
       <c r="G38" s="140"/>
@@ -4946,16 +4973,16 @@
       <c r="B39" s="77" t="s">
         <v>265</v>
       </c>
-      <c r="C39" s="185" t="s">
+      <c r="C39" s="146" t="s">
         <v>144</v>
       </c>
-      <c r="D39" s="189">
+      <c r="D39" s="150">
         <v>45712</v>
       </c>
-      <c r="E39" s="190" t="s">
+      <c r="E39" s="151" t="s">
         <v>268</v>
       </c>
-      <c r="F39" s="187">
+      <c r="F39" s="148">
         <v>0.5</v>
       </c>
       <c r="G39" s="140"/>
@@ -4999,26 +5026,26 @@
       <c r="B40" s="77" t="s">
         <v>266</v>
       </c>
-      <c r="C40" s="185" t="s">
+      <c r="C40" s="146" t="s">
         <v>144</v>
       </c>
-      <c r="D40" s="189">
+      <c r="D40" s="150">
         <v>45712</v>
       </c>
-      <c r="E40" s="190" t="s">
+      <c r="E40" s="151" t="s">
         <v>263</v>
       </c>
-      <c r="F40" s="187">
+      <c r="F40" s="148">
         <v>0.5</v>
       </c>
       <c r="G40" s="140"/>
       <c r="H40" s="2"/>
-      <c r="I40" s="145"/>
-      <c r="J40" s="146"/>
-      <c r="K40" s="146"/>
-      <c r="L40" s="146"/>
-      <c r="M40" s="146"/>
-      <c r="N40" s="147"/>
+      <c r="I40" s="174"/>
+      <c r="J40" s="175"/>
+      <c r="K40" s="175"/>
+      <c r="L40" s="175"/>
+      <c r="M40" s="175"/>
+      <c r="N40" s="176"/>
       <c r="O40" s="2"/>
       <c r="P40" s="2"/>
       <c r="Q40" s="2"/>
@@ -5052,16 +5079,16 @@
       <c r="B41" s="77" t="s">
         <v>267</v>
       </c>
-      <c r="C41" s="185" t="s">
+      <c r="C41" s="146" t="s">
         <v>146</v>
       </c>
-      <c r="D41" s="189">
+      <c r="D41" s="150">
         <v>45712</v>
       </c>
-      <c r="E41" s="190" t="s">
+      <c r="E41" s="151" t="s">
         <v>269</v>
       </c>
-      <c r="F41" s="187">
+      <c r="F41" s="148">
         <v>0.5</v>
       </c>
       <c r="G41" s="140"/>
@@ -5105,16 +5132,16 @@
       <c r="B42" s="77" t="s">
         <v>270</v>
       </c>
-      <c r="C42" s="185" t="s">
+      <c r="C42" s="146" t="s">
         <v>145</v>
       </c>
-      <c r="D42" s="189">
+      <c r="D42" s="150">
         <v>45713</v>
       </c>
-      <c r="E42" s="190" t="s">
+      <c r="E42" s="151" t="s">
         <v>271</v>
       </c>
-      <c r="F42" s="187">
+      <c r="F42" s="148">
         <v>0.5</v>
       </c>
       <c r="G42" s="140"/>
@@ -5158,16 +5185,16 @@
       <c r="B43" s="77" t="s">
         <v>272</v>
       </c>
-      <c r="C43" s="185" t="s">
+      <c r="C43" s="146" t="s">
         <v>144</v>
       </c>
-      <c r="D43" s="189">
+      <c r="D43" s="150">
         <v>45713</v>
       </c>
-      <c r="E43" s="190" t="s">
+      <c r="E43" s="151" t="s">
         <v>273</v>
       </c>
-      <c r="F43" s="187">
+      <c r="F43" s="148">
         <v>0.5</v>
       </c>
       <c r="G43" s="140"/>
@@ -5211,16 +5238,16 @@
       <c r="B44" s="77" t="s">
         <v>274</v>
       </c>
-      <c r="C44" s="185" t="s">
+      <c r="C44" s="146" t="s">
         <v>144</v>
       </c>
-      <c r="D44" s="189">
+      <c r="D44" s="150">
         <v>45713</v>
       </c>
-      <c r="E44" s="190" t="s">
+      <c r="E44" s="151" t="s">
         <v>271</v>
       </c>
-      <c r="F44" s="187">
+      <c r="F44" s="148">
         <v>0.5</v>
       </c>
       <c r="G44" s="140"/>
@@ -5264,16 +5291,16 @@
       <c r="B45" s="77" t="s">
         <v>275</v>
       </c>
-      <c r="C45" s="185" t="s">
+      <c r="C45" s="146" t="s">
         <v>144</v>
       </c>
-      <c r="D45" s="189">
+      <c r="D45" s="150">
         <v>45803</v>
       </c>
-      <c r="E45" s="190" t="s">
+      <c r="E45" s="151" t="s">
         <v>276</v>
       </c>
-      <c r="F45" s="191">
+      <c r="F45" s="152">
         <v>0.5</v>
       </c>
       <c r="G45" s="140"/>
@@ -5317,16 +5344,16 @@
       <c r="B46" s="77" t="s">
         <v>277</v>
       </c>
-      <c r="C46" s="185" t="s">
+      <c r="C46" s="146" t="s">
         <v>144</v>
       </c>
-      <c r="D46" s="189">
+      <c r="D46" s="150">
         <v>45714</v>
       </c>
-      <c r="E46" s="190" t="s">
+      <c r="E46" s="151" t="s">
         <v>271</v>
       </c>
-      <c r="F46" s="187">
+      <c r="F46" s="148">
         <v>0.5</v>
       </c>
       <c r="G46" s="140"/>
@@ -5370,16 +5397,16 @@
       <c r="B47" s="77" t="s">
         <v>278</v>
       </c>
-      <c r="C47" s="185" t="s">
+      <c r="C47" s="146" t="s">
         <v>145</v>
       </c>
-      <c r="D47" s="189">
+      <c r="D47" s="150">
         <v>45723</v>
       </c>
-      <c r="E47" s="190" t="s">
+      <c r="E47" s="151" t="s">
         <v>271</v>
       </c>
-      <c r="F47" s="187">
+      <c r="F47" s="148">
         <v>1</v>
       </c>
       <c r="G47" s="140"/>
@@ -5423,14 +5450,14 @@
       <c r="B48" s="77" t="s">
         <v>281</v>
       </c>
-      <c r="C48" s="185"/>
-      <c r="D48" s="192">
+      <c r="C48" s="146"/>
+      <c r="D48" s="153">
         <v>45726</v>
       </c>
-      <c r="E48" s="190" t="s">
+      <c r="E48" s="151" t="s">
         <v>282</v>
       </c>
-      <c r="F48" s="187">
+      <c r="F48" s="148">
         <v>0.5</v>
       </c>
       <c r="G48" s="140"/>
@@ -5474,11 +5501,11 @@
       <c r="B49" s="77" t="s">
         <v>283</v>
       </c>
-      <c r="C49" s="185"/>
-      <c r="D49" s="192">
+      <c r="C49" s="146"/>
+      <c r="D49" s="153">
         <v>45743</v>
       </c>
-      <c r="E49" s="190" t="s">
+      <c r="E49" s="151" t="s">
         <v>284</v>
       </c>
       <c r="F49" s="142">
@@ -5525,13 +5552,13 @@
       <c r="B50" s="78" t="s">
         <v>285</v>
       </c>
-      <c r="C50" s="185" t="s">
+      <c r="C50" s="146" t="s">
         <v>144</v>
       </c>
-      <c r="D50" s="192">
+      <c r="D50" s="153">
         <v>45805</v>
       </c>
-      <c r="E50" s="190" t="s">
+      <c r="E50" s="151" t="s">
         <v>271</v>
       </c>
       <c r="F50" s="142">
@@ -5578,11 +5605,11 @@
       <c r="B51" s="74" t="s">
         <v>286</v>
       </c>
-      <c r="C51" s="185"/>
-      <c r="D51" s="192">
+      <c r="C51" s="146"/>
+      <c r="D51" s="153">
         <v>45806</v>
       </c>
-      <c r="E51" s="190" t="s">
+      <c r="E51" s="151" t="s">
         <v>295</v>
       </c>
       <c r="F51" s="142">
@@ -5629,11 +5656,11 @@
       <c r="B52" s="74" t="s">
         <v>287</v>
       </c>
-      <c r="C52" s="185"/>
-      <c r="D52" s="192">
+      <c r="C52" s="146"/>
+      <c r="D52" s="153">
         <v>45793</v>
       </c>
-      <c r="E52" s="190" t="s">
+      <c r="E52" s="151" t="s">
         <v>302</v>
       </c>
       <c r="F52" s="142">
@@ -5680,11 +5707,11 @@
       <c r="B53" s="74" t="s">
         <v>288</v>
       </c>
-      <c r="C53" s="185"/>
-      <c r="D53" s="192">
+      <c r="C53" s="146"/>
+      <c r="D53" s="153">
         <v>45855</v>
       </c>
-      <c r="E53" s="190" t="s">
+      <c r="E53" s="151" t="s">
         <v>296</v>
       </c>
       <c r="F53" s="142">
@@ -5731,11 +5758,11 @@
       <c r="B54" s="74" t="s">
         <v>303</v>
       </c>
-      <c r="C54" s="185"/>
-      <c r="D54" s="192">
+      <c r="C54" s="146"/>
+      <c r="D54" s="153">
         <v>45859</v>
       </c>
-      <c r="E54" s="190" t="s">
+      <c r="E54" s="151" t="s">
         <v>304</v>
       </c>
       <c r="F54" s="142">
@@ -5782,11 +5809,11 @@
       <c r="B55" s="74" t="s">
         <v>305</v>
       </c>
-      <c r="C55" s="185"/>
-      <c r="D55" s="192">
+      <c r="C55" s="146"/>
+      <c r="D55" s="153">
         <v>45866</v>
       </c>
-      <c r="E55" s="190" t="s">
+      <c r="E55" s="151" t="s">
         <v>306</v>
       </c>
       <c r="F55" s="142">
@@ -5833,11 +5860,11 @@
       <c r="B56" s="74" t="s">
         <v>289</v>
       </c>
-      <c r="C56" s="185"/>
-      <c r="D56" s="192">
+      <c r="C56" s="146"/>
+      <c r="D56" s="153">
         <v>45873</v>
       </c>
-      <c r="E56" s="190" t="s">
+      <c r="E56" s="151" t="s">
         <v>297</v>
       </c>
       <c r="F56" s="142">
@@ -5884,11 +5911,11 @@
       <c r="B57" s="74" t="s">
         <v>290</v>
       </c>
-      <c r="C57" s="185"/>
-      <c r="D57" s="192">
+      <c r="C57" s="146"/>
+      <c r="D57" s="153">
         <v>45873</v>
       </c>
-      <c r="E57" s="190" t="s">
+      <c r="E57" s="151" t="s">
         <v>297</v>
       </c>
       <c r="F57" s="142">
@@ -5932,14 +5959,14 @@
     </row>
     <row r="58" spans="1:41" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A58" s="3"/>
-      <c r="B58" s="190" t="s">
+      <c r="B58" s="151" t="s">
         <v>291</v>
       </c>
-      <c r="C58" s="185"/>
-      <c r="D58" s="192">
+      <c r="C58" s="146"/>
+      <c r="D58" s="153">
         <v>45874</v>
       </c>
-      <c r="E58" s="190" t="s">
+      <c r="E58" s="151" t="s">
         <v>298</v>
       </c>
       <c r="F58" s="142">
@@ -5983,14 +6010,14 @@
     </row>
     <row r="59" spans="1:41" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A59" s="3"/>
-      <c r="B59" s="190" t="s">
+      <c r="B59" s="151" t="s">
         <v>292</v>
       </c>
-      <c r="C59" s="185"/>
-      <c r="D59" s="192">
+      <c r="C59" s="146"/>
+      <c r="D59" s="153">
         <v>45880</v>
       </c>
-      <c r="E59" s="190" t="s">
+      <c r="E59" s="151" t="s">
         <v>299</v>
       </c>
       <c r="F59" s="142">
@@ -6034,14 +6061,14 @@
     </row>
     <row r="60" spans="1:41" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A60" s="3"/>
-      <c r="B60" s="190" t="s">
+      <c r="B60" s="151" t="s">
         <v>293</v>
       </c>
-      <c r="C60" s="185"/>
-      <c r="D60" s="192">
+      <c r="C60" s="146"/>
+      <c r="D60" s="153">
         <v>45884</v>
       </c>
-      <c r="E60" s="190" t="s">
+      <c r="E60" s="151" t="s">
         <v>300</v>
       </c>
       <c r="F60" s="142">
@@ -6085,14 +6112,14 @@
     </row>
     <row r="61" spans="1:41" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A61" s="3"/>
-      <c r="B61" s="190" t="s">
+      <c r="B61" s="151" t="s">
         <v>294</v>
       </c>
-      <c r="C61" s="185"/>
-      <c r="D61" s="192">
+      <c r="C61" s="146"/>
+      <c r="D61" s="153">
         <v>45888</v>
       </c>
-      <c r="E61" s="190" t="s">
+      <c r="E61" s="151" t="s">
         <v>301</v>
       </c>
       <c r="F61" s="142">
@@ -6136,14 +6163,14 @@
     </row>
     <row r="62" spans="1:41" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="3"/>
-      <c r="B62" s="190" t="s">
+      <c r="B62" s="151" t="s">
         <v>307</v>
       </c>
-      <c r="C62" s="185"/>
-      <c r="D62" s="192">
+      <c r="C62" s="146"/>
+      <c r="D62" s="153">
         <v>45960</v>
       </c>
-      <c r="E62" s="190" t="s">
+      <c r="E62" s="151" t="s">
         <v>300</v>
       </c>
       <c r="F62" s="142">
@@ -6187,14 +6214,14 @@
     </row>
     <row r="63" spans="1:41" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A63" s="3"/>
-      <c r="B63" s="190" t="s">
+      <c r="B63" s="151" t="s">
         <v>308</v>
       </c>
-      <c r="C63" s="185"/>
-      <c r="D63" s="192">
+      <c r="C63" s="146"/>
+      <c r="D63" s="153">
         <v>45966</v>
       </c>
-      <c r="E63" s="190" t="s">
+      <c r="E63" s="151" t="s">
         <v>309</v>
       </c>
       <c r="F63" s="142">
@@ -6238,14 +6265,14 @@
     </row>
     <row r="64" spans="1:41" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A64" s="3"/>
-      <c r="B64" s="190" t="s">
+      <c r="B64" s="151" t="s">
         <v>310</v>
       </c>
-      <c r="C64" s="185"/>
-      <c r="D64" s="192">
+      <c r="C64" s="146"/>
+      <c r="D64" s="153">
         <v>45978</v>
       </c>
-      <c r="E64" s="190" t="s">
+      <c r="E64" s="151" t="s">
         <v>315</v>
       </c>
       <c r="F64" s="142">
@@ -6289,14 +6316,14 @@
     </row>
     <row r="65" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A65" s="3"/>
-      <c r="B65" s="190" t="s">
+      <c r="B65" s="151" t="s">
         <v>312</v>
       </c>
-      <c r="C65" s="185"/>
-      <c r="D65" s="192">
+      <c r="C65" s="146"/>
+      <c r="D65" s="153">
         <v>46031</v>
       </c>
-      <c r="E65" s="193" t="s">
+      <c r="E65" s="154" t="s">
         <v>318</v>
       </c>
       <c r="F65" s="142">
@@ -6340,14 +6367,14 @@
     </row>
     <row r="66" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A66" s="3"/>
-      <c r="B66" s="190" t="s">
+      <c r="B66" s="151" t="s">
         <v>311</v>
       </c>
-      <c r="C66" s="185"/>
-      <c r="D66" s="192">
+      <c r="C66" s="146"/>
+      <c r="D66" s="153">
         <v>46037</v>
       </c>
-      <c r="E66" s="190" t="s">
+      <c r="E66" s="151" t="s">
         <v>316</v>
       </c>
       <c r="F66" s="142">
@@ -6391,14 +6418,14 @@
     </row>
     <row r="67" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="3"/>
-      <c r="B67" s="190" t="s">
+      <c r="B67" s="151" t="s">
         <v>314</v>
       </c>
-      <c r="C67" s="185"/>
-      <c r="D67" s="192">
+      <c r="C67" s="146"/>
+      <c r="D67" s="153">
         <v>46056</v>
       </c>
-      <c r="E67" s="193" t="s">
+      <c r="E67" s="154" t="s">
         <v>317</v>
       </c>
       <c r="F67" s="142">
@@ -6442,14 +6469,14 @@
     </row>
     <row r="68" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A68" s="3"/>
-      <c r="B68" s="190" t="s">
+      <c r="B68" s="151" t="s">
         <v>313</v>
       </c>
-      <c r="C68" s="185"/>
-      <c r="D68" s="192">
+      <c r="C68" s="146"/>
+      <c r="D68" s="153">
         <v>46052</v>
       </c>
-      <c r="E68" s="193" t="s">
+      <c r="E68" s="154" t="s">
         <v>319</v>
       </c>
       <c r="F68" s="142">
@@ -6493,13 +6520,21 @@
     </row>
     <row r="69" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="3"/>
-      <c r="B69" s="190"/>
-      <c r="C69" s="185"/>
-      <c r="D69" s="190"/>
-      <c r="E69" s="194"/>
-      <c r="F69" s="195"/>
-      <c r="G69" s="142"/>
-      <c r="H69" s="140"/>
+      <c r="B69" s="151" t="s">
+        <v>321</v>
+      </c>
+      <c r="C69" s="146"/>
+      <c r="D69" s="153">
+        <v>46129</v>
+      </c>
+      <c r="E69" s="154" t="s">
+        <v>319</v>
+      </c>
+      <c r="F69" s="142">
+        <v>1</v>
+      </c>
+      <c r="G69" s="140"/>
+      <c r="H69" s="2"/>
       <c r="I69" s="2"/>
       <c r="J69" s="2"/>
       <c r="K69" s="2"/>
@@ -6533,22 +6568,24 @@
       <c r="AM69" s="2"/>
       <c r="AN69" s="2"/>
       <c r="AO69" s="2"/>
-      <c r="AP69" s="2"/>
-    </row>
-    <row r="70" spans="1:42" x14ac:dyDescent="0.25">
+    </row>
+    <row r="70" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="3"/>
-      <c r="B70" s="196" t="s">
-        <v>7</v>
-      </c>
-      <c r="C70" s="197"/>
-      <c r="D70" s="198"/>
-      <c r="E70" s="199"/>
-      <c r="F70" s="199"/>
-      <c r="G70" s="200">
-        <f>SUM(G36:G69)</f>
-        <v>0</v>
-      </c>
-      <c r="H70" s="141"/>
+      <c r="B70" s="151" t="s">
+        <v>322</v>
+      </c>
+      <c r="C70" s="146"/>
+      <c r="D70" s="153">
+        <v>46122</v>
+      </c>
+      <c r="E70" s="154" t="s">
+        <v>316</v>
+      </c>
+      <c r="F70" s="142">
+        <v>2</v>
+      </c>
+      <c r="G70" s="140"/>
+      <c r="H70" s="2"/>
       <c r="I70" s="2"/>
       <c r="J70" s="2"/>
       <c r="K70" s="2"/>
@@ -6582,17 +6619,24 @@
       <c r="AM70" s="2"/>
       <c r="AN70" s="2"/>
       <c r="AO70" s="2"/>
-      <c r="AP70" s="2"/>
-    </row>
-    <row r="71" spans="1:42" x14ac:dyDescent="0.25">
+    </row>
+    <row r="71" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="3"/>
-      <c r="B71" s="201"/>
-      <c r="C71" s="202"/>
-      <c r="D71" s="203"/>
-      <c r="E71" s="177"/>
-      <c r="F71" s="177"/>
-      <c r="G71" s="204"/>
-      <c r="H71" s="122"/>
+      <c r="B71" s="151" t="s">
+        <v>324</v>
+      </c>
+      <c r="C71" s="146"/>
+      <c r="D71" s="153">
+        <v>46072</v>
+      </c>
+      <c r="E71" s="154" t="s">
+        <v>323</v>
+      </c>
+      <c r="F71" s="142">
+        <v>7</v>
+      </c>
+      <c r="G71" s="140"/>
+      <c r="H71" s="2"/>
       <c r="I71" s="2"/>
       <c r="J71" s="2"/>
       <c r="K71" s="2"/>
@@ -6626,22 +6670,24 @@
       <c r="AM71" s="2"/>
       <c r="AN71" s="2"/>
       <c r="AO71" s="2"/>
-      <c r="AP71" s="2"/>
-    </row>
-    <row r="72" spans="1:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    </row>
+    <row r="72" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A72" s="3"/>
-      <c r="B72" s="205" t="s">
-        <v>40</v>
-      </c>
-      <c r="C72" s="205"/>
-      <c r="D72" s="206"/>
-      <c r="E72" s="207"/>
-      <c r="F72" s="207"/>
-      <c r="G72" s="208">
-        <f>G70+G19+G28+G71</f>
-        <v>352</v>
-      </c>
-      <c r="H72" s="42"/>
+      <c r="B72" s="151" t="s">
+        <v>320</v>
+      </c>
+      <c r="C72" s="146"/>
+      <c r="D72" s="153">
+        <v>46127</v>
+      </c>
+      <c r="E72" s="154" t="s">
+        <v>319</v>
+      </c>
+      <c r="F72" s="142">
+        <v>1</v>
+      </c>
+      <c r="G72" s="140"/>
+      <c r="H72" s="2"/>
       <c r="I72" s="2"/>
       <c r="J72" s="2"/>
       <c r="K72" s="2"/>
@@ -6675,17 +6721,16 @@
       <c r="AM72" s="2"/>
       <c r="AN72" s="2"/>
       <c r="AO72" s="2"/>
-      <c r="AP72" s="2"/>
-    </row>
-    <row r="73" spans="1:42" x14ac:dyDescent="0.25">
+    </row>
+    <row r="73" spans="1:42" ht="17.25" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="3"/>
-      <c r="B73" s="2"/>
-      <c r="C73" s="2"/>
-      <c r="D73" s="2"/>
-      <c r="E73" s="2"/>
-      <c r="F73" s="2"/>
-      <c r="G73" s="2"/>
-      <c r="H73" s="41"/>
+      <c r="B73" s="151"/>
+      <c r="C73" s="146"/>
+      <c r="D73" s="151"/>
+      <c r="E73" s="168"/>
+      <c r="F73" s="169"/>
+      <c r="G73" s="142"/>
+      <c r="H73" s="140"/>
       <c r="I73" s="2"/>
       <c r="J73" s="2"/>
       <c r="K73" s="2"/>
@@ -6723,11 +6768,18 @@
     </row>
     <row r="74" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A74" s="3"/>
-      <c r="B74" s="1"/>
-      <c r="D74" s="2"/>
-      <c r="F74" s="2"/>
-      <c r="G74" s="2"/>
-      <c r="H74" s="35"/>
+      <c r="B74" s="155" t="s">
+        <v>7</v>
+      </c>
+      <c r="C74" s="156"/>
+      <c r="D74" s="157"/>
+      <c r="E74" s="170"/>
+      <c r="F74" s="170"/>
+      <c r="G74" s="158">
+        <f>SUM(G36:G73)</f>
+        <v>0</v>
+      </c>
+      <c r="H74" s="141"/>
       <c r="I74" s="2"/>
       <c r="J74" s="2"/>
       <c r="K74" s="2"/>
@@ -6765,17 +6817,13 @@
     </row>
     <row r="75" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A75" s="3"/>
-      <c r="B75" s="55" t="s">
-        <v>41</v>
-      </c>
-      <c r="C75" s="55">
-        <f>'List - Hide'!AC11</f>
-        <v>487</v>
-      </c>
-      <c r="D75" s="2"/>
-      <c r="F75" s="2"/>
-      <c r="G75" s="2"/>
-      <c r="H75" s="35"/>
+      <c r="B75" s="159"/>
+      <c r="C75" s="160"/>
+      <c r="D75" s="161"/>
+      <c r="E75" s="143"/>
+      <c r="F75" s="143"/>
+      <c r="G75" s="162"/>
+      <c r="H75" s="122"/>
       <c r="I75" s="2"/>
       <c r="J75" s="2"/>
       <c r="K75" s="2"/>
@@ -6811,19 +6859,20 @@
       <c r="AO75" s="2"/>
       <c r="AP75" s="2"/>
     </row>
-    <row r="76" spans="1:42" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:42" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A76" s="3"/>
-      <c r="B76" s="55" t="s">
-        <v>42</v>
-      </c>
-      <c r="C76" s="55">
-        <f>G72</f>
-        <v>352</v>
-      </c>
-      <c r="D76" s="2"/>
-      <c r="F76" s="2"/>
-      <c r="G76" s="2"/>
-      <c r="H76" s="35"/>
+      <c r="B76" s="163" t="s">
+        <v>40</v>
+      </c>
+      <c r="C76" s="163"/>
+      <c r="D76" s="164"/>
+      <c r="E76" s="165"/>
+      <c r="F76" s="165"/>
+      <c r="G76" s="166">
+        <f>G74+G19+G28+G75</f>
+        <v>489</v>
+      </c>
+      <c r="H76" s="42"/>
       <c r="I76" s="2"/>
       <c r="J76" s="2"/>
       <c r="K76" s="2"/>
@@ -6861,17 +6910,13 @@
     </row>
     <row r="77" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A77" s="3"/>
-      <c r="B77" s="55" t="s">
-        <v>43</v>
-      </c>
-      <c r="C77" s="57">
-        <f>C75-C76</f>
-        <v>135</v>
-      </c>
+      <c r="B77" s="2"/>
+      <c r="C77" s="2"/>
       <c r="D77" s="2"/>
+      <c r="E77" s="2"/>
       <c r="F77" s="2"/>
       <c r="G77" s="2"/>
-      <c r="H77" s="35"/>
+      <c r="H77" s="41"/>
       <c r="I77" s="2"/>
       <c r="J77" s="2"/>
       <c r="K77" s="2"/>
@@ -6909,7 +6954,7 @@
     </row>
     <row r="78" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A78" s="3"/>
-      <c r="B78" s="2"/>
+      <c r="B78" s="1"/>
       <c r="D78" s="2"/>
       <c r="F78" s="2"/>
       <c r="G78" s="2"/>
@@ -6951,11 +6996,17 @@
     </row>
     <row r="79" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A79" s="3"/>
-      <c r="B79" s="2"/>
+      <c r="B79" s="55" t="s">
+        <v>41</v>
+      </c>
+      <c r="C79" s="55">
+        <f>'List - Hide'!AC11</f>
+        <v>487</v>
+      </c>
       <c r="D79" s="2"/>
       <c r="F79" s="2"/>
       <c r="G79" s="2"/>
-      <c r="H79" s="2"/>
+      <c r="H79" s="35"/>
       <c r="I79" s="2"/>
       <c r="J79" s="2"/>
       <c r="K79" s="2"/>
@@ -6993,11 +7044,17 @@
     </row>
     <row r="80" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A80" s="3"/>
-      <c r="B80" s="2"/>
+      <c r="B80" s="55" t="s">
+        <v>42</v>
+      </c>
+      <c r="C80" s="55">
+        <f>G76</f>
+        <v>489</v>
+      </c>
       <c r="D80" s="2"/>
       <c r="F80" s="2"/>
       <c r="G80" s="2"/>
-      <c r="H80" s="2"/>
+      <c r="H80" s="35"/>
       <c r="I80" s="2"/>
       <c r="J80" s="2"/>
       <c r="K80" s="2"/>
@@ -7035,13 +7092,17 @@
     </row>
     <row r="81" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A81" s="3"/>
-      <c r="B81" s="2"/>
-      <c r="C81" s="2"/>
+      <c r="B81" s="55" t="s">
+        <v>43</v>
+      </c>
+      <c r="C81" s="57">
+        <f>C79-C80</f>
+        <v>-2</v>
+      </c>
       <c r="D81" s="2"/>
-      <c r="E81" s="2"/>
       <c r="F81" s="2"/>
       <c r="G81" s="2"/>
-      <c r="H81" s="2"/>
+      <c r="H81" s="35"/>
       <c r="I81" s="2"/>
       <c r="J81" s="2"/>
       <c r="K81" s="2"/>
@@ -7080,12 +7141,10 @@
     <row r="82" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A82" s="3"/>
       <c r="B82" s="2"/>
-      <c r="C82" s="2"/>
       <c r="D82" s="2"/>
-      <c r="E82" s="2"/>
       <c r="F82" s="2"/>
       <c r="G82" s="2"/>
-      <c r="H82" s="2"/>
+      <c r="H82" s="35"/>
       <c r="I82" s="2"/>
       <c r="J82" s="2"/>
       <c r="K82" s="2"/>
@@ -7124,9 +7183,7 @@
     <row r="83" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A83" s="3"/>
       <c r="B83" s="2"/>
-      <c r="C83" s="2"/>
       <c r="D83" s="2"/>
-      <c r="E83" s="2"/>
       <c r="F83" s="2"/>
       <c r="G83" s="2"/>
       <c r="H83" s="2"/>
@@ -7168,9 +7225,7 @@
     <row r="84" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A84" s="3"/>
       <c r="B84" s="2"/>
-      <c r="C84" s="2"/>
       <c r="D84" s="2"/>
-      <c r="E84" s="2"/>
       <c r="F84" s="2"/>
       <c r="G84" s="2"/>
       <c r="H84" s="2"/>
@@ -7218,7 +7273,7 @@
       <c r="F85" s="2"/>
       <c r="G85" s="2"/>
       <c r="H85" s="2"/>
-      <c r="I85" s="4"/>
+      <c r="I85" s="2"/>
       <c r="J85" s="2"/>
       <c r="K85" s="2"/>
       <c r="L85" s="2"/>
@@ -7262,7 +7317,7 @@
       <c r="F86" s="2"/>
       <c r="G86" s="2"/>
       <c r="H86" s="2"/>
-      <c r="I86" s="5"/>
+      <c r="I86" s="2"/>
       <c r="J86" s="2"/>
       <c r="K86" s="2"/>
       <c r="L86" s="2"/>
@@ -7298,7 +7353,7 @@
       <c r="AP86" s="2"/>
     </row>
     <row r="87" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="A87" s="2"/>
+      <c r="A87" s="3"/>
       <c r="B87" s="2"/>
       <c r="C87" s="2"/>
       <c r="D87" s="2"/>
@@ -7306,7 +7361,7 @@
       <c r="F87" s="2"/>
       <c r="G87" s="2"/>
       <c r="H87" s="2"/>
-      <c r="I87" s="5"/>
+      <c r="I87" s="2"/>
       <c r="J87" s="2"/>
       <c r="K87" s="2"/>
       <c r="L87" s="2"/>
@@ -7342,7 +7397,7 @@
       <c r="AP87" s="2"/>
     </row>
     <row r="88" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="A88" s="2"/>
+      <c r="A88" s="3"/>
       <c r="B88" s="2"/>
       <c r="C88" s="2"/>
       <c r="D88" s="2"/>
@@ -7386,7 +7441,7 @@
       <c r="AP88" s="2"/>
     </row>
     <row r="89" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="A89" s="2"/>
+      <c r="A89" s="3"/>
       <c r="B89" s="2"/>
       <c r="C89" s="2"/>
       <c r="D89" s="2"/>
@@ -7394,7 +7449,7 @@
       <c r="F89" s="2"/>
       <c r="G89" s="2"/>
       <c r="H89" s="2"/>
-      <c r="I89" s="2"/>
+      <c r="I89" s="4"/>
       <c r="J89" s="2"/>
       <c r="K89" s="2"/>
       <c r="L89" s="2"/>
@@ -7430,7 +7485,7 @@
       <c r="AP89" s="2"/>
     </row>
     <row r="90" spans="1:42" x14ac:dyDescent="0.25">
-      <c r="A90" s="2"/>
+      <c r="A90" s="3"/>
       <c r="B90" s="2"/>
       <c r="C90" s="2"/>
       <c r="D90" s="2"/>
@@ -7438,7 +7493,7 @@
       <c r="F90" s="2"/>
       <c r="G90" s="2"/>
       <c r="H90" s="2"/>
-      <c r="I90" s="2"/>
+      <c r="I90" s="5"/>
       <c r="J90" s="2"/>
       <c r="K90" s="2"/>
       <c r="L90" s="2"/>
@@ -7482,7 +7537,7 @@
       <c r="F91" s="2"/>
       <c r="G91" s="2"/>
       <c r="H91" s="2"/>
-      <c r="I91" s="2"/>
+      <c r="I91" s="5"/>
       <c r="J91" s="2"/>
       <c r="K91" s="2"/>
       <c r="L91" s="2"/>
@@ -7729,8 +7784,15 @@
       <c r="AG96" s="2"/>
       <c r="AH96" s="2"/>
       <c r="AI96" s="2"/>
-    </row>
-    <row r="97" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ96" s="2"/>
+      <c r="AK96" s="2"/>
+      <c r="AL96" s="2"/>
+      <c r="AM96" s="2"/>
+      <c r="AN96" s="2"/>
+      <c r="AO96" s="2"/>
+      <c r="AP96" s="2"/>
+    </row>
+    <row r="97" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A97" s="2"/>
       <c r="B97" s="2"/>
       <c r="C97" s="2"/>
@@ -7766,8 +7828,15 @@
       <c r="AG97" s="2"/>
       <c r="AH97" s="2"/>
       <c r="AI97" s="2"/>
-    </row>
-    <row r="98" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ97" s="2"/>
+      <c r="AK97" s="2"/>
+      <c r="AL97" s="2"/>
+      <c r="AM97" s="2"/>
+      <c r="AN97" s="2"/>
+      <c r="AO97" s="2"/>
+      <c r="AP97" s="2"/>
+    </row>
+    <row r="98" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A98" s="2"/>
       <c r="B98" s="2"/>
       <c r="C98" s="2"/>
@@ -7803,8 +7872,15 @@
       <c r="AG98" s="2"/>
       <c r="AH98" s="2"/>
       <c r="AI98" s="2"/>
-    </row>
-    <row r="99" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ98" s="2"/>
+      <c r="AK98" s="2"/>
+      <c r="AL98" s="2"/>
+      <c r="AM98" s="2"/>
+      <c r="AN98" s="2"/>
+      <c r="AO98" s="2"/>
+      <c r="AP98" s="2"/>
+    </row>
+    <row r="99" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A99" s="2"/>
       <c r="B99" s="2"/>
       <c r="C99" s="2"/>
@@ -7840,8 +7916,15 @@
       <c r="AG99" s="2"/>
       <c r="AH99" s="2"/>
       <c r="AI99" s="2"/>
-    </row>
-    <row r="100" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="AJ99" s="2"/>
+      <c r="AK99" s="2"/>
+      <c r="AL99" s="2"/>
+      <c r="AM99" s="2"/>
+      <c r="AN99" s="2"/>
+      <c r="AO99" s="2"/>
+      <c r="AP99" s="2"/>
+    </row>
+    <row r="100" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A100" s="2"/>
       <c r="B100" s="2"/>
       <c r="C100" s="2"/>
@@ -7878,7 +7961,7 @@
       <c r="AH100" s="2"/>
       <c r="AI100" s="2"/>
     </row>
-    <row r="101" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="101" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A101" s="2"/>
       <c r="B101" s="2"/>
       <c r="C101" s="2"/>
@@ -7915,7 +7998,7 @@
       <c r="AH101" s="2"/>
       <c r="AI101" s="2"/>
     </row>
-    <row r="102" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="102" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A102" s="2"/>
       <c r="B102" s="2"/>
       <c r="C102" s="2"/>
@@ -7952,7 +8035,7 @@
       <c r="AH102" s="2"/>
       <c r="AI102" s="2"/>
     </row>
-    <row r="103" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="103" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A103" s="2"/>
       <c r="B103" s="2"/>
       <c r="C103" s="2"/>
@@ -7989,7 +8072,7 @@
       <c r="AH103" s="2"/>
       <c r="AI103" s="2"/>
     </row>
-    <row r="104" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="104" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A104" s="2"/>
       <c r="B104" s="2"/>
       <c r="C104" s="2"/>
@@ -8026,7 +8109,7 @@
       <c r="AH104" s="2"/>
       <c r="AI104" s="2"/>
     </row>
-    <row r="105" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="105" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A105" s="2"/>
       <c r="B105" s="2"/>
       <c r="C105" s="2"/>
@@ -8063,7 +8146,7 @@
       <c r="AH105" s="2"/>
       <c r="AI105" s="2"/>
     </row>
-    <row r="106" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="106" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A106" s="2"/>
       <c r="B106" s="2"/>
       <c r="C106" s="2"/>
@@ -8100,7 +8183,7 @@
       <c r="AH106" s="2"/>
       <c r="AI106" s="2"/>
     </row>
-    <row r="107" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="107" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A107" s="2"/>
       <c r="B107" s="2"/>
       <c r="C107" s="2"/>
@@ -8137,7 +8220,7 @@
       <c r="AH107" s="2"/>
       <c r="AI107" s="2"/>
     </row>
-    <row r="108" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="108" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A108" s="2"/>
       <c r="B108" s="2"/>
       <c r="C108" s="2"/>
@@ -8174,7 +8257,7 @@
       <c r="AH108" s="2"/>
       <c r="AI108" s="2"/>
     </row>
-    <row r="109" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="109" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A109" s="2"/>
       <c r="B109" s="2"/>
       <c r="C109" s="2"/>
@@ -8211,7 +8294,7 @@
       <c r="AH109" s="2"/>
       <c r="AI109" s="2"/>
     </row>
-    <row r="110" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="110" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A110" s="2"/>
       <c r="B110" s="2"/>
       <c r="C110" s="2"/>
@@ -8248,7 +8331,7 @@
       <c r="AH110" s="2"/>
       <c r="AI110" s="2"/>
     </row>
-    <row r="111" spans="1:35" x14ac:dyDescent="0.25">
+    <row r="111" spans="1:42" x14ac:dyDescent="0.25">
       <c r="A111" s="2"/>
       <c r="B111" s="2"/>
       <c r="C111" s="2"/>
@@ -8285,8 +8368,8 @@
       <c r="AH111" s="2"/>
       <c r="AI111" s="2"/>
     </row>
-    <row r="112" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A112" s="3"/>
+    <row r="112" spans="1:42" x14ac:dyDescent="0.25">
+      <c r="A112" s="2"/>
       <c r="B112" s="2"/>
       <c r="C112" s="2"/>
       <c r="D112" s="2"/>
@@ -8323,7 +8406,7 @@
       <c r="AI112" s="2"/>
     </row>
     <row r="113" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A113" s="3"/>
+      <c r="A113" s="2"/>
       <c r="B113" s="2"/>
       <c r="C113" s="2"/>
       <c r="D113" s="2"/>
@@ -8360,7 +8443,7 @@
       <c r="AI113" s="2"/>
     </row>
     <row r="114" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A114" s="3"/>
+      <c r="A114" s="2"/>
       <c r="B114" s="2"/>
       <c r="C114" s="2"/>
       <c r="D114" s="2"/>
@@ -8397,7 +8480,7 @@
       <c r="AI114" s="2"/>
     </row>
     <row r="115" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A115" s="3"/>
+      <c r="A115" s="2"/>
       <c r="B115" s="2"/>
       <c r="C115" s="2"/>
       <c r="D115" s="2"/>
@@ -8434,6 +8517,7 @@
       <c r="AI115" s="2"/>
     </row>
     <row r="116" spans="1:35" x14ac:dyDescent="0.25">
+      <c r="A116" s="3"/>
       <c r="B116" s="2"/>
       <c r="C116" s="2"/>
       <c r="D116" s="2"/>
@@ -8470,7 +8554,7 @@
       <c r="AI116" s="2"/>
     </row>
     <row r="117" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A117" s="4"/>
+      <c r="A117" s="3"/>
       <c r="B117" s="2"/>
       <c r="C117" s="2"/>
       <c r="D117" s="2"/>
@@ -8507,7 +8591,7 @@
       <c r="AI117" s="2"/>
     </row>
     <row r="118" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A118" s="2"/>
+      <c r="A118" s="3"/>
       <c r="B118" s="2"/>
       <c r="C118" s="2"/>
       <c r="D118" s="2"/>
@@ -8544,7 +8628,7 @@
       <c r="AI118" s="2"/>
     </row>
     <row r="119" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A119" s="2"/>
+      <c r="A119" s="3"/>
       <c r="B119" s="2"/>
       <c r="C119" s="2"/>
       <c r="D119" s="2"/>
@@ -8581,7 +8665,6 @@
       <c r="AI119" s="2"/>
     </row>
     <row r="120" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A120" s="2"/>
       <c r="B120" s="2"/>
       <c r="C120" s="2"/>
       <c r="D120" s="2"/>
@@ -8618,7 +8701,7 @@
       <c r="AI120" s="2"/>
     </row>
     <row r="121" spans="1:35" x14ac:dyDescent="0.25">
-      <c r="A121" s="2"/>
+      <c r="A121" s="4"/>
       <c r="B121" s="2"/>
       <c r="C121" s="2"/>
       <c r="D121" s="2"/>
@@ -9783,6 +9866,23 @@
       <c r="P152" s="2"/>
       <c r="Q152" s="2"/>
       <c r="R152" s="2"/>
+      <c r="S152" s="2"/>
+      <c r="T152" s="2"/>
+      <c r="U152" s="2"/>
+      <c r="V152" s="2"/>
+      <c r="W152" s="2"/>
+      <c r="X152" s="2"/>
+      <c r="Y152" s="2"/>
+      <c r="Z152" s="2"/>
+      <c r="AA152" s="2"/>
+      <c r="AB152" s="2"/>
+      <c r="AC152" s="2"/>
+      <c r="AD152" s="2"/>
+      <c r="AE152" s="2"/>
+      <c r="AF152" s="2"/>
+      <c r="AG152" s="2"/>
+      <c r="AH152" s="2"/>
+      <c r="AI152" s="2"/>
     </row>
     <row r="153" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A153" s="2"/>
@@ -9803,6 +9903,23 @@
       <c r="P153" s="2"/>
       <c r="Q153" s="2"/>
       <c r="R153" s="2"/>
+      <c r="S153" s="2"/>
+      <c r="T153" s="2"/>
+      <c r="U153" s="2"/>
+      <c r="V153" s="2"/>
+      <c r="W153" s="2"/>
+      <c r="X153" s="2"/>
+      <c r="Y153" s="2"/>
+      <c r="Z153" s="2"/>
+      <c r="AA153" s="2"/>
+      <c r="AB153" s="2"/>
+      <c r="AC153" s="2"/>
+      <c r="AD153" s="2"/>
+      <c r="AE153" s="2"/>
+      <c r="AF153" s="2"/>
+      <c r="AG153" s="2"/>
+      <c r="AH153" s="2"/>
+      <c r="AI153" s="2"/>
     </row>
     <row r="154" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A154" s="2"/>
@@ -9823,6 +9940,23 @@
       <c r="P154" s="2"/>
       <c r="Q154" s="2"/>
       <c r="R154" s="2"/>
+      <c r="S154" s="2"/>
+      <c r="T154" s="2"/>
+      <c r="U154" s="2"/>
+      <c r="V154" s="2"/>
+      <c r="W154" s="2"/>
+      <c r="X154" s="2"/>
+      <c r="Y154" s="2"/>
+      <c r="Z154" s="2"/>
+      <c r="AA154" s="2"/>
+      <c r="AB154" s="2"/>
+      <c r="AC154" s="2"/>
+      <c r="AD154" s="2"/>
+      <c r="AE154" s="2"/>
+      <c r="AF154" s="2"/>
+      <c r="AG154" s="2"/>
+      <c r="AH154" s="2"/>
+      <c r="AI154" s="2"/>
     </row>
     <row r="155" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A155" s="2"/>
@@ -9843,6 +9977,23 @@
       <c r="P155" s="2"/>
       <c r="Q155" s="2"/>
       <c r="R155" s="2"/>
+      <c r="S155" s="2"/>
+      <c r="T155" s="2"/>
+      <c r="U155" s="2"/>
+      <c r="V155" s="2"/>
+      <c r="W155" s="2"/>
+      <c r="X155" s="2"/>
+      <c r="Y155" s="2"/>
+      <c r="Z155" s="2"/>
+      <c r="AA155" s="2"/>
+      <c r="AB155" s="2"/>
+      <c r="AC155" s="2"/>
+      <c r="AD155" s="2"/>
+      <c r="AE155" s="2"/>
+      <c r="AF155" s="2"/>
+      <c r="AG155" s="2"/>
+      <c r="AH155" s="2"/>
+      <c r="AI155" s="2"/>
     </row>
     <row r="156" spans="1:35" x14ac:dyDescent="0.25">
       <c r="A156" s="2"/>
@@ -12316,6 +12467,13 @@
       <c r="I279" s="2"/>
       <c r="J279" s="2"/>
       <c r="K279" s="2"/>
+      <c r="L279" s="2"/>
+      <c r="M279" s="2"/>
+      <c r="N279" s="2"/>
+      <c r="O279" s="2"/>
+      <c r="P279" s="2"/>
+      <c r="Q279" s="2"/>
+      <c r="R279" s="2"/>
     </row>
     <row r="280" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A280" s="2"/>
@@ -12329,6 +12487,13 @@
       <c r="I280" s="2"/>
       <c r="J280" s="2"/>
       <c r="K280" s="2"/>
+      <c r="L280" s="2"/>
+      <c r="M280" s="2"/>
+      <c r="N280" s="2"/>
+      <c r="O280" s="2"/>
+      <c r="P280" s="2"/>
+      <c r="Q280" s="2"/>
+      <c r="R280" s="2"/>
     </row>
     <row r="281" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A281" s="2"/>
@@ -12342,6 +12507,13 @@
       <c r="I281" s="2"/>
       <c r="J281" s="2"/>
       <c r="K281" s="2"/>
+      <c r="L281" s="2"/>
+      <c r="M281" s="2"/>
+      <c r="N281" s="2"/>
+      <c r="O281" s="2"/>
+      <c r="P281" s="2"/>
+      <c r="Q281" s="2"/>
+      <c r="R281" s="2"/>
     </row>
     <row r="282" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A282" s="2"/>
@@ -12355,6 +12527,13 @@
       <c r="I282" s="2"/>
       <c r="J282" s="2"/>
       <c r="K282" s="2"/>
+      <c r="L282" s="2"/>
+      <c r="M282" s="2"/>
+      <c r="N282" s="2"/>
+      <c r="O282" s="2"/>
+      <c r="P282" s="2"/>
+      <c r="Q282" s="2"/>
+      <c r="R282" s="2"/>
     </row>
     <row r="283" spans="1:18" x14ac:dyDescent="0.25">
       <c r="A283" s="2"/>
@@ -12644,6 +12823,12 @@
     </row>
     <row r="305" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A305" s="2"/>
+      <c r="B305" s="2"/>
+      <c r="C305" s="2"/>
+      <c r="D305" s="2"/>
+      <c r="E305" s="2"/>
+      <c r="F305" s="2"/>
+      <c r="G305" s="2"/>
       <c r="H305" s="2"/>
       <c r="I305" s="2"/>
       <c r="J305" s="2"/>
@@ -12651,6 +12836,12 @@
     </row>
     <row r="306" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A306" s="2"/>
+      <c r="B306" s="2"/>
+      <c r="C306" s="2"/>
+      <c r="D306" s="2"/>
+      <c r="E306" s="2"/>
+      <c r="F306" s="2"/>
+      <c r="G306" s="2"/>
       <c r="H306" s="2"/>
       <c r="I306" s="2"/>
       <c r="J306" s="2"/>
@@ -12658,6 +12849,12 @@
     </row>
     <row r="307" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A307" s="2"/>
+      <c r="B307" s="2"/>
+      <c r="C307" s="2"/>
+      <c r="D307" s="2"/>
+      <c r="E307" s="2"/>
+      <c r="F307" s="2"/>
+      <c r="G307" s="2"/>
       <c r="H307" s="2"/>
       <c r="I307" s="2"/>
       <c r="J307" s="2"/>
@@ -12665,24 +12862,34 @@
     </row>
     <row r="308" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A308" s="2"/>
+      <c r="B308" s="2"/>
+      <c r="C308" s="2"/>
+      <c r="D308" s="2"/>
+      <c r="E308" s="2"/>
+      <c r="F308" s="2"/>
+      <c r="G308" s="2"/>
+      <c r="H308" s="2"/>
       <c r="I308" s="2"/>
       <c r="J308" s="2"/>
       <c r="K308" s="2"/>
     </row>
     <row r="309" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A309" s="2"/>
+      <c r="H309" s="2"/>
       <c r="I309" s="2"/>
       <c r="J309" s="2"/>
       <c r="K309" s="2"/>
     </row>
     <row r="310" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A310" s="2"/>
+      <c r="H310" s="2"/>
       <c r="I310" s="2"/>
       <c r="J310" s="2"/>
       <c r="K310" s="2"/>
     </row>
     <row r="311" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A311" s="2"/>
+      <c r="H311" s="2"/>
       <c r="I311" s="2"/>
       <c r="J311" s="2"/>
       <c r="K311" s="2"/>
@@ -12747,11 +12954,35 @@
       <c r="J321" s="2"/>
       <c r="K321" s="2"/>
     </row>
+    <row r="322" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A322" s="2"/>
+      <c r="I322" s="2"/>
+      <c r="J322" s="2"/>
+      <c r="K322" s="2"/>
+    </row>
+    <row r="323" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A323" s="2"/>
+      <c r="I323" s="2"/>
+      <c r="J323" s="2"/>
+      <c r="K323" s="2"/>
+    </row>
+    <row r="324" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A324" s="2"/>
+      <c r="I324" s="2"/>
+      <c r="J324" s="2"/>
+      <c r="K324" s="2"/>
+    </row>
+    <row r="325" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A325" s="2"/>
+      <c r="I325" s="2"/>
+      <c r="J325" s="2"/>
+      <c r="K325" s="2"/>
+    </row>
   </sheetData>
   <mergeCells count="16">
     <mergeCell ref="H22:H28"/>
-    <mergeCell ref="E69:F69"/>
-    <mergeCell ref="E70:F70"/>
+    <mergeCell ref="E73:F73"/>
+    <mergeCell ref="E74:F74"/>
     <mergeCell ref="J2:O2"/>
     <mergeCell ref="J29:O29"/>
     <mergeCell ref="J17:O17"/>
@@ -12790,13 +13021,13 @@
           <x14:formula1>
             <xm:f>'List - Hide'!$A$2:$A$17</xm:f>
           </x14:formula1>
-          <xm:sqref>C70:C71 C81:C99 C73</xm:sqref>
+          <xm:sqref>C74:C75 C85:C103 C77</xm:sqref>
         </x14:dataValidation>
         <x14:dataValidation type="list" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid Entry!" error="Please pick from the list!" prompt="Please select from the list" xr:uid="{00000000-0002-0000-0000-000007000000}">
           <x14:formula1>
             <xm:f>'List - Hide'!$C$2:$C$19</xm:f>
           </x14:formula1>
-          <xm:sqref>C36:C69</xm:sqref>
+          <xm:sqref>C36:C73</xm:sqref>
         </x14:dataValidation>
       </x14:dataValidations>
     </ext>
@@ -26453,10 +26684,10 @@
       <c r="AH1" s="64"/>
     </row>
     <row r="2" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="168" t="s">
+      <c r="A2" s="194" t="s">
         <v>142</v>
       </c>
-      <c r="B2" s="172">
+      <c r="B2" s="198">
         <v>1</v>
       </c>
       <c r="C2" s="68" t="s">
@@ -26512,8 +26743,8 @@
       <c r="AH2" s="65"/>
     </row>
     <row r="3" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A3" s="169"/>
-      <c r="B3" s="166"/>
+      <c r="A3" s="195"/>
+      <c r="B3" s="192"/>
       <c r="C3" s="70" t="s">
         <v>144</v>
       </c>
@@ -26564,8 +26795,8 @@
       <c r="AH3" s="65"/>
     </row>
     <row r="4" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A4" s="169"/>
-      <c r="B4" s="166"/>
+      <c r="A4" s="195"/>
+      <c r="B4" s="192"/>
       <c r="C4" s="70" t="s">
         <v>145</v>
       </c>
@@ -26616,8 +26847,8 @@
       <c r="AH4" s="65"/>
     </row>
     <row r="5" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="169"/>
-      <c r="B5" s="171"/>
+      <c r="A5" s="195"/>
+      <c r="B5" s="197"/>
       <c r="C5" s="70" t="s">
         <v>146</v>
       </c>
@@ -26668,8 +26899,8 @@
       <c r="AH5" s="65"/>
     </row>
     <row r="6" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A6" s="169"/>
-      <c r="B6" s="166">
+      <c r="A6" s="195"/>
+      <c r="B6" s="192">
         <v>2</v>
       </c>
       <c r="C6" s="70" t="s">
@@ -26724,8 +26955,8 @@
       <c r="AH6" s="65"/>
     </row>
     <row r="7" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A7" s="169"/>
-      <c r="B7" s="166"/>
+      <c r="A7" s="195"/>
+      <c r="B7" s="192"/>
       <c r="C7" s="70" t="s">
         <v>148</v>
       </c>
@@ -26776,8 +27007,8 @@
       <c r="AH7" s="65"/>
     </row>
     <row r="8" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A8" s="169"/>
-      <c r="B8" s="166"/>
+      <c r="A8" s="195"/>
+      <c r="B8" s="192"/>
       <c r="C8" s="70" t="s">
         <v>149</v>
       </c>
@@ -26827,8 +27058,8 @@
       <c r="AH8" s="65"/>
     </row>
     <row r="9" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A9" s="169"/>
-      <c r="B9" s="166"/>
+      <c r="A9" s="195"/>
+      <c r="B9" s="192"/>
       <c r="C9" s="70" t="s">
         <v>150</v>
       </c>
@@ -26883,8 +27114,8 @@
       <c r="AH9" s="65"/>
     </row>
     <row r="10" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A10" s="169"/>
-      <c r="B10" s="166">
+      <c r="A10" s="195"/>
+      <c r="B10" s="192">
         <v>3</v>
       </c>
       <c r="C10" s="70" t="s">
@@ -26942,8 +27173,8 @@
       <c r="AH10" s="65"/>
     </row>
     <row r="11" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A11" s="169"/>
-      <c r="B11" s="166"/>
+      <c r="A11" s="195"/>
+      <c r="B11" s="192"/>
       <c r="C11" s="70" t="s">
         <v>155</v>
       </c>
@@ -26998,8 +27229,8 @@
       <c r="AH11" s="65"/>
     </row>
     <row r="12" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A12" s="169"/>
-      <c r="B12" s="166"/>
+      <c r="A12" s="195"/>
+      <c r="B12" s="192"/>
       <c r="C12" s="70" t="s">
         <v>157</v>
       </c>
@@ -27057,8 +27288,8 @@
       <c r="AH12" s="65"/>
     </row>
     <row r="13" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A13" s="169"/>
-      <c r="B13" s="166"/>
+      <c r="A13" s="195"/>
+      <c r="B13" s="192"/>
       <c r="C13" s="70" t="s">
         <v>162</v>
       </c>
@@ -27124,8 +27355,8 @@
       <c r="AH13" s="65"/>
     </row>
     <row r="14" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A14" s="169"/>
-      <c r="B14" s="166">
+      <c r="A14" s="195"/>
+      <c r="B14" s="192">
         <v>4</v>
       </c>
       <c r="C14" s="70" t="s">
@@ -27192,8 +27423,8 @@
       <c r="AH14" s="65"/>
     </row>
     <row r="15" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A15" s="169"/>
-      <c r="B15" s="166"/>
+      <c r="A15" s="195"/>
+      <c r="B15" s="192"/>
       <c r="C15" s="70" t="s">
         <v>165</v>
       </c>
@@ -27256,8 +27487,8 @@
       <c r="AH15" s="65"/>
     </row>
     <row r="16" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A16" s="169"/>
-      <c r="B16" s="166"/>
+      <c r="A16" s="195"/>
+      <c r="B16" s="192"/>
       <c r="C16" s="70" t="s">
         <v>166</v>
       </c>
@@ -27320,8 +27551,8 @@
       <c r="AH16" s="65"/>
     </row>
     <row r="17" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A17" s="169"/>
-      <c r="B17" s="166"/>
+      <c r="A17" s="195"/>
+      <c r="B17" s="192"/>
       <c r="C17" s="70" t="s">
         <v>167</v>
       </c>
@@ -27384,8 +27615,8 @@
       <c r="AH17" s="65"/>
     </row>
     <row r="18" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A18" s="169"/>
-      <c r="B18" s="166">
+      <c r="A18" s="195"/>
+      <c r="B18" s="192">
         <v>5</v>
       </c>
       <c r="C18" s="70" t="s">
@@ -27452,8 +27683,8 @@
       <c r="AH18" s="65"/>
     </row>
     <row r="19" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A19" s="169"/>
-      <c r="B19" s="166"/>
+      <c r="A19" s="195"/>
+      <c r="B19" s="192"/>
       <c r="C19" s="70" t="s">
         <v>169</v>
       </c>
@@ -27517,8 +27748,8 @@
       <c r="AH19" s="65"/>
     </row>
     <row r="20" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A20" s="169"/>
-      <c r="B20" s="166"/>
+      <c r="A20" s="195"/>
+      <c r="B20" s="192"/>
       <c r="C20" s="70" t="s">
         <v>170</v>
       </c>
@@ -27581,8 +27812,8 @@
       <c r="AH20" s="65"/>
     </row>
     <row r="21" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A21" s="169"/>
-      <c r="B21" s="166"/>
+      <c r="A21" s="195"/>
+      <c r="B21" s="192"/>
       <c r="C21" s="70" t="s">
         <v>171</v>
       </c>
@@ -27645,8 +27876,8 @@
       <c r="AG21" s="80"/>
     </row>
     <row r="22" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A22" s="169"/>
-      <c r="B22" s="166">
+      <c r="A22" s="195"/>
+      <c r="B22" s="192">
         <v>6</v>
       </c>
       <c r="C22" s="70" t="s">
@@ -27712,8 +27943,8 @@
       <c r="AG22" s="80"/>
     </row>
     <row r="23" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A23" s="169"/>
-      <c r="B23" s="166"/>
+      <c r="A23" s="195"/>
+      <c r="B23" s="192"/>
       <c r="C23" s="70" t="s">
         <v>173</v>
       </c>
@@ -27778,8 +28009,8 @@
       <c r="AG23" s="80"/>
     </row>
     <row r="24" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A24" s="169"/>
-      <c r="B24" s="166"/>
+      <c r="A24" s="195"/>
+      <c r="B24" s="192"/>
       <c r="C24" s="70" t="s">
         <v>174</v>
       </c>
@@ -27840,8 +28071,8 @@
       <c r="AG24" s="80"/>
     </row>
     <row r="25" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A25" s="169"/>
-      <c r="B25" s="166"/>
+      <c r="A25" s="195"/>
+      <c r="B25" s="192"/>
       <c r="C25" s="70" t="s">
         <v>175</v>
       </c>
@@ -27899,8 +28130,8 @@
       <c r="AG25" s="65"/>
     </row>
     <row r="26" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A26" s="169"/>
-      <c r="B26" s="166">
+      <c r="A26" s="195"/>
+      <c r="B26" s="192">
         <v>7</v>
       </c>
       <c r="C26" s="70" t="s">
@@ -27960,8 +28191,8 @@
       <c r="AG26" s="65"/>
     </row>
     <row r="27" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A27" s="169"/>
-      <c r="B27" s="166"/>
+      <c r="A27" s="195"/>
+      <c r="B27" s="192"/>
       <c r="C27" s="70" t="s">
         <v>177</v>
       </c>
@@ -28017,8 +28248,8 @@
       </c>
     </row>
     <row r="28" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A28" s="169"/>
-      <c r="B28" s="166"/>
+      <c r="A28" s="195"/>
+      <c r="B28" s="192"/>
       <c r="C28" s="70" t="s">
         <v>179</v>
       </c>
@@ -28074,8 +28305,8 @@
       </c>
     </row>
     <row r="29" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A29" s="169"/>
-      <c r="B29" s="166"/>
+      <c r="A29" s="195"/>
+      <c r="B29" s="192"/>
       <c r="C29" s="70" t="s">
         <v>181</v>
       </c>
@@ -28132,8 +28363,8 @@
       </c>
     </row>
     <row r="30" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A30" s="169"/>
-      <c r="B30" s="166">
+      <c r="A30" s="195"/>
+      <c r="B30" s="192">
         <v>8</v>
       </c>
       <c r="C30" s="70" t="s">
@@ -28191,8 +28422,8 @@
       </c>
     </row>
     <row r="31" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A31" s="169"/>
-      <c r="B31" s="166"/>
+      <c r="A31" s="195"/>
+      <c r="B31" s="192"/>
       <c r="C31" s="70" t="s">
         <v>186</v>
       </c>
@@ -28247,8 +28478,8 @@
       </c>
     </row>
     <row r="32" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A32" s="169"/>
-      <c r="B32" s="166"/>
+      <c r="A32" s="195"/>
+      <c r="B32" s="192"/>
       <c r="C32" s="70" t="s">
         <v>188</v>
       </c>
@@ -28298,8 +28529,8 @@
       </c>
     </row>
     <row r="33" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A33" s="169"/>
-      <c r="B33" s="166"/>
+      <c r="A33" s="195"/>
+      <c r="B33" s="192"/>
       <c r="C33" s="70" t="s">
         <v>189</v>
       </c>
@@ -28345,8 +28576,8 @@
       <c r="AA33" s="65"/>
     </row>
     <row r="34" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A34" s="169"/>
-      <c r="B34" s="166">
+      <c r="A34" s="195"/>
+      <c r="B34" s="192">
         <v>9</v>
       </c>
       <c r="C34" s="70" t="s">
@@ -28392,8 +28623,8 @@
       <c r="AA34" s="65"/>
     </row>
     <row r="35" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A35" s="169"/>
-      <c r="B35" s="166"/>
+      <c r="A35" s="195"/>
+      <c r="B35" s="192"/>
       <c r="C35" s="70" t="s">
         <v>191</v>
       </c>
@@ -28436,8 +28667,8 @@
       <c r="AA35" s="65"/>
     </row>
     <row r="36" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A36" s="169"/>
-      <c r="B36" s="166"/>
+      <c r="A36" s="195"/>
+      <c r="B36" s="192"/>
       <c r="C36" s="70" t="s">
         <v>192</v>
       </c>
@@ -28482,8 +28713,8 @@
       <c r="AA36" s="65"/>
     </row>
     <row r="37" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A37" s="169"/>
-      <c r="B37" s="166"/>
+      <c r="A37" s="195"/>
+      <c r="B37" s="192"/>
       <c r="C37" s="70" t="s">
         <v>193</v>
       </c>
@@ -28526,8 +28757,8 @@
       <c r="AA37" s="65"/>
     </row>
     <row r="38" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A38" s="169"/>
-      <c r="B38" s="166">
+      <c r="A38" s="195"/>
+      <c r="B38" s="192">
         <v>10</v>
       </c>
       <c r="C38" s="70" t="s">
@@ -28575,8 +28806,8 @@
       <c r="AH38" s="65"/>
     </row>
     <row r="39" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A39" s="169"/>
-      <c r="B39" s="166"/>
+      <c r="A39" s="195"/>
+      <c r="B39" s="192"/>
       <c r="C39" s="70" t="s">
         <v>195</v>
       </c>
@@ -28621,8 +28852,8 @@
       <c r="AH39" s="65"/>
     </row>
     <row r="40" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A40" s="169"/>
-      <c r="B40" s="166"/>
+      <c r="A40" s="195"/>
+      <c r="B40" s="192"/>
       <c r="C40" s="70" t="s">
         <v>196</v>
       </c>
@@ -28666,8 +28897,8 @@
       <c r="AH40" s="65"/>
     </row>
     <row r="41" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A41" s="169"/>
-      <c r="B41" s="166"/>
+      <c r="A41" s="195"/>
+      <c r="B41" s="192"/>
       <c r="C41" s="70" t="s">
         <v>197</v>
       </c>
@@ -28717,8 +28948,8 @@
       <c r="AH41" s="65"/>
     </row>
     <row r="42" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A42" s="169"/>
-      <c r="B42" s="166">
+      <c r="A42" s="195"/>
+      <c r="B42" s="192">
         <v>11</v>
       </c>
       <c r="C42" s="70" t="s">
@@ -28771,8 +29002,8 @@
       <c r="AH42" s="65"/>
     </row>
     <row r="43" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A43" s="169"/>
-      <c r="B43" s="166"/>
+      <c r="A43" s="195"/>
+      <c r="B43" s="192"/>
       <c r="C43" s="70" t="s">
         <v>199</v>
       </c>
@@ -28825,8 +29056,8 @@
       <c r="AH43" s="65"/>
     </row>
     <row r="44" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A44" s="169"/>
-      <c r="B44" s="166"/>
+      <c r="A44" s="195"/>
+      <c r="B44" s="192"/>
       <c r="C44" s="70" t="s">
         <v>200</v>
       </c>
@@ -28876,8 +29107,8 @@
       <c r="AH44" s="65"/>
     </row>
     <row r="45" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A45" s="169"/>
-      <c r="B45" s="166"/>
+      <c r="A45" s="195"/>
+      <c r="B45" s="192"/>
       <c r="C45" s="70" t="s">
         <v>201</v>
       </c>
@@ -28927,8 +29158,8 @@
       <c r="AH45" s="65"/>
     </row>
     <row r="46" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A46" s="169"/>
-      <c r="B46" s="166">
+      <c r="A46" s="195"/>
+      <c r="B46" s="192">
         <v>12</v>
       </c>
       <c r="C46" s="70" t="s">
@@ -28982,8 +29213,8 @@
       <c r="AH46" s="65"/>
     </row>
     <row r="47" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A47" s="169"/>
-      <c r="B47" s="166"/>
+      <c r="A47" s="195"/>
+      <c r="B47" s="192"/>
       <c r="C47" s="70" t="s">
         <v>203</v>
       </c>
@@ -29033,8 +29264,8 @@
       <c r="AH47" s="65"/>
     </row>
     <row r="48" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A48" s="169"/>
-      <c r="B48" s="166"/>
+      <c r="A48" s="195"/>
+      <c r="B48" s="192"/>
       <c r="C48" s="70" t="s">
         <v>204</v>
       </c>
@@ -29086,8 +29317,8 @@
       <c r="AH48" s="65"/>
     </row>
     <row r="49" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A49" s="169"/>
-      <c r="B49" s="166"/>
+      <c r="A49" s="195"/>
+      <c r="B49" s="192"/>
       <c r="C49" s="70" t="s">
         <v>205</v>
       </c>
@@ -29137,8 +29368,8 @@
       <c r="AH49" s="65"/>
     </row>
     <row r="50" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A50" s="169"/>
-      <c r="B50" s="166">
+      <c r="A50" s="195"/>
+      <c r="B50" s="192">
         <v>13</v>
       </c>
       <c r="C50" s="70" t="s">
@@ -29192,8 +29423,8 @@
       <c r="AH50" s="65"/>
     </row>
     <row r="51" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A51" s="169"/>
-      <c r="B51" s="166"/>
+      <c r="A51" s="195"/>
+      <c r="B51" s="192"/>
       <c r="C51" s="70" t="s">
         <v>207</v>
       </c>
@@ -29243,8 +29474,8 @@
       <c r="AH51" s="65"/>
     </row>
     <row r="52" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A52" s="169"/>
-      <c r="B52" s="166"/>
+      <c r="A52" s="195"/>
+      <c r="B52" s="192"/>
       <c r="C52" s="70" t="s">
         <v>208</v>
       </c>
@@ -29293,8 +29524,8 @@
       <c r="AH52" s="65"/>
     </row>
     <row r="53" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A53" s="169"/>
-      <c r="B53" s="166"/>
+      <c r="A53" s="195"/>
+      <c r="B53" s="192"/>
       <c r="C53" s="70" t="s">
         <v>209</v>
       </c>
@@ -29344,8 +29575,8 @@
       <c r="AH53" s="65"/>
     </row>
     <row r="54" spans="1:34" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="169"/>
-      <c r="B54" s="166">
+      <c r="A54" s="195"/>
+      <c r="B54" s="192">
         <v>14</v>
       </c>
       <c r="C54" s="70" t="s">
@@ -29399,8 +29630,8 @@
       <c r="AH54" s="65"/>
     </row>
     <row r="55" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A55" s="169"/>
-      <c r="B55" s="166"/>
+      <c r="A55" s="195"/>
+      <c r="B55" s="192"/>
       <c r="C55" s="70" t="s">
         <v>211</v>
       </c>
@@ -29451,8 +29682,8 @@
       <c r="AH55" s="65"/>
     </row>
     <row r="56" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A56" s="169"/>
-      <c r="B56" s="166"/>
+      <c r="A56" s="195"/>
+      <c r="B56" s="192"/>
       <c r="C56" s="70" t="s">
         <v>212</v>
       </c>
@@ -29502,8 +29733,8 @@
       <c r="AH56" s="65"/>
     </row>
     <row r="57" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A57" s="169"/>
-      <c r="B57" s="166"/>
+      <c r="A57" s="195"/>
+      <c r="B57" s="192"/>
       <c r="C57" s="70" t="s">
         <v>213</v>
       </c>
@@ -29554,8 +29785,8 @@
       <c r="AH57" s="65"/>
     </row>
     <row r="58" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A58" s="169"/>
-      <c r="B58" s="166">
+      <c r="A58" s="195"/>
+      <c r="B58" s="192">
         <v>15</v>
       </c>
       <c r="C58" s="70" t="s">
@@ -29610,8 +29841,8 @@
       <c r="AH58" s="65"/>
     </row>
     <row r="59" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A59" s="169"/>
-      <c r="B59" s="166"/>
+      <c r="A59" s="195"/>
+      <c r="B59" s="192"/>
       <c r="C59" s="70" t="s">
         <v>215</v>
       </c>
@@ -29662,8 +29893,8 @@
       <c r="AH59" s="65"/>
     </row>
     <row r="60" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A60" s="169"/>
-      <c r="B60" s="166"/>
+      <c r="A60" s="195"/>
+      <c r="B60" s="192"/>
       <c r="C60" s="70" t="s">
         <v>216</v>
       </c>
@@ -29714,8 +29945,8 @@
       <c r="AH60" s="65"/>
     </row>
     <row r="61" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A61" s="170"/>
-      <c r="B61" s="167"/>
+      <c r="A61" s="196"/>
+      <c r="B61" s="193"/>
       <c r="C61" s="72" t="s">
         <v>217</v>
       </c>
@@ -29766,10 +29997,10 @@
       <c r="AH61" s="65"/>
     </row>
     <row r="62" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A62" s="168" t="s">
+      <c r="A62" s="194" t="s">
         <v>136</v>
       </c>
-      <c r="B62" s="171">
+      <c r="B62" s="197">
         <v>16</v>
       </c>
       <c r="C62" s="70" t="s">
@@ -29821,8 +30052,8 @@
       <c r="AH62" s="65"/>
     </row>
     <row r="63" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A63" s="169"/>
-      <c r="B63" s="166"/>
+      <c r="A63" s="195"/>
+      <c r="B63" s="192"/>
       <c r="C63" s="70" t="s">
         <v>219</v>
       </c>
@@ -29872,8 +30103,8 @@
       <c r="AH63" s="65"/>
     </row>
     <row r="64" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A64" s="169"/>
-      <c r="B64" s="166"/>
+      <c r="A64" s="195"/>
+      <c r="B64" s="192"/>
       <c r="C64" s="70" t="s">
         <v>220</v>
       </c>
@@ -29923,8 +30154,8 @@
       <c r="AH64" s="65"/>
     </row>
     <row r="65" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A65" s="169"/>
-      <c r="B65" s="166"/>
+      <c r="A65" s="195"/>
+      <c r="B65" s="192"/>
       <c r="C65" s="70" t="s">
         <v>221</v>
       </c>
@@ -29974,8 +30205,8 @@
       <c r="AH65" s="65"/>
     </row>
     <row r="66" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A66" s="169"/>
-      <c r="B66" s="166">
+      <c r="A66" s="195"/>
+      <c r="B66" s="192">
         <v>17</v>
       </c>
       <c r="C66" s="70" t="s">
@@ -30027,8 +30258,8 @@
       <c r="AH66" s="65"/>
     </row>
     <row r="67" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A67" s="169"/>
-      <c r="B67" s="166"/>
+      <c r="A67" s="195"/>
+      <c r="B67" s="192"/>
       <c r="C67" s="70" t="s">
         <v>223</v>
       </c>
@@ -30078,8 +30309,8 @@
       <c r="AH67" s="65"/>
     </row>
     <row r="68" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A68" s="169"/>
-      <c r="B68" s="166"/>
+      <c r="A68" s="195"/>
+      <c r="B68" s="192"/>
       <c r="C68" s="70" t="s">
         <v>224</v>
       </c>
@@ -30129,8 +30360,8 @@
       <c r="AH68" s="65"/>
     </row>
     <row r="69" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A69" s="169"/>
-      <c r="B69" s="166"/>
+      <c r="A69" s="195"/>
+      <c r="B69" s="192"/>
       <c r="C69" s="70" t="s">
         <v>225</v>
       </c>
@@ -30180,8 +30411,8 @@
       <c r="AH69" s="65"/>
     </row>
     <row r="70" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A70" s="169"/>
-      <c r="B70" s="166">
+      <c r="A70" s="195"/>
+      <c r="B70" s="192">
         <v>18</v>
       </c>
       <c r="C70" s="70" t="s">
@@ -30233,8 +30464,8 @@
       <c r="AH70" s="65"/>
     </row>
     <row r="71" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A71" s="169"/>
-      <c r="B71" s="166"/>
+      <c r="A71" s="195"/>
+      <c r="B71" s="192"/>
       <c r="C71" s="70" t="s">
         <v>227</v>
       </c>
@@ -30284,8 +30515,8 @@
       <c r="AH71" s="65"/>
     </row>
     <row r="72" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A72" s="169"/>
-      <c r="B72" s="166"/>
+      <c r="A72" s="195"/>
+      <c r="B72" s="192"/>
       <c r="C72" s="70" t="s">
         <v>228</v>
       </c>
@@ -30335,8 +30566,8 @@
       <c r="AH72" s="65"/>
     </row>
     <row r="73" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A73" s="169"/>
-      <c r="B73" s="166"/>
+      <c r="A73" s="195"/>
+      <c r="B73" s="192"/>
       <c r="C73" s="70" t="s">
         <v>229</v>
       </c>
@@ -30386,8 +30617,8 @@
       <c r="AH73" s="65"/>
     </row>
     <row r="74" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A74" s="169"/>
-      <c r="B74" s="166">
+      <c r="A74" s="195"/>
+      <c r="B74" s="192">
         <v>19</v>
       </c>
       <c r="C74" s="70" t="s">
@@ -30439,8 +30670,8 @@
       <c r="AH74" s="65"/>
     </row>
     <row r="75" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A75" s="169"/>
-      <c r="B75" s="166"/>
+      <c r="A75" s="195"/>
+      <c r="B75" s="192"/>
       <c r="C75" s="70" t="s">
         <v>231</v>
       </c>
@@ -30490,8 +30721,8 @@
       <c r="AH75" s="65"/>
     </row>
     <row r="76" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A76" s="169"/>
-      <c r="B76" s="166"/>
+      <c r="A76" s="195"/>
+      <c r="B76" s="192"/>
       <c r="C76" s="70" t="s">
         <v>232</v>
       </c>
@@ -30541,8 +30772,8 @@
       <c r="AH76" s="65"/>
     </row>
     <row r="77" spans="1:34" x14ac:dyDescent="0.25">
-      <c r="A77" s="170"/>
-      <c r="B77" s="167"/>
+      <c r="A77" s="196"/>
+      <c r="B77" s="193"/>
       <c r="C77" s="72" t="s">
         <v>233</v>
       </c>
@@ -30729,10 +30960,10 @@
     <row r="80" spans="1:34" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A80" s="65"/>
       <c r="B80" s="65"/>
-      <c r="C80" s="162" t="s">
+      <c r="C80" s="201" t="s">
         <v>234</v>
       </c>
-      <c r="D80" s="163"/>
+      <c r="D80" s="202"/>
       <c r="E80" s="69">
         <v>60</v>
       </c>
@@ -30771,10 +31002,10 @@
     <row r="81" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A81" s="65"/>
       <c r="B81" s="65"/>
-      <c r="C81" s="164" t="s">
+      <c r="C81" s="203" t="s">
         <v>236</v>
       </c>
-      <c r="D81" s="165"/>
+      <c r="D81" s="204"/>
       <c r="E81" s="71">
         <v>322.5</v>
       </c>
@@ -30811,10 +31042,10 @@
     <row r="82" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A82" s="65"/>
       <c r="B82" s="65"/>
-      <c r="C82" s="164" t="s">
+      <c r="C82" s="203" t="s">
         <v>237</v>
       </c>
-      <c r="D82" s="165"/>
+      <c r="D82" s="204"/>
       <c r="E82" s="71">
         <v>35</v>
       </c>
@@ -30851,10 +31082,10 @@
     <row r="83" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A83" s="65"/>
       <c r="B83" s="65"/>
-      <c r="C83" s="164" t="s">
+      <c r="C83" s="203" t="s">
         <v>238</v>
       </c>
-      <c r="D83" s="165"/>
+      <c r="D83" s="204"/>
       <c r="E83" s="71">
         <v>287</v>
       </c>
@@ -30891,10 +31122,10 @@
     <row r="84" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A84" s="65"/>
       <c r="B84" s="65"/>
-      <c r="C84" s="164" t="s">
+      <c r="C84" s="203" t="s">
         <v>239</v>
       </c>
-      <c r="D84" s="165"/>
+      <c r="D84" s="204"/>
       <c r="E84" s="71">
         <v>60</v>
       </c>
@@ -30931,10 +31162,10 @@
     <row r="85" spans="1:34" x14ac:dyDescent="0.25">
       <c r="A85" s="65"/>
       <c r="B85" s="65"/>
-      <c r="C85" s="160" t="s">
+      <c r="C85" s="199" t="s">
         <v>240</v>
       </c>
-      <c r="D85" s="161"/>
+      <c r="D85" s="200"/>
       <c r="E85" s="73">
         <f>Y79</f>
         <v>483</v>
@@ -31002,6 +31233,17 @@
     </row>
   </sheetData>
   <mergeCells count="27">
+    <mergeCell ref="C85:D85"/>
+    <mergeCell ref="C80:D80"/>
+    <mergeCell ref="C81:D81"/>
+    <mergeCell ref="C82:D82"/>
+    <mergeCell ref="C83:D83"/>
+    <mergeCell ref="C84:D84"/>
+    <mergeCell ref="B22:B25"/>
+    <mergeCell ref="B26:B29"/>
+    <mergeCell ref="B30:B33"/>
+    <mergeCell ref="B34:B37"/>
+    <mergeCell ref="B38:B41"/>
     <mergeCell ref="B66:B69"/>
     <mergeCell ref="B70:B73"/>
     <mergeCell ref="B74:B77"/>
@@ -31018,17 +31260,6 @@
     <mergeCell ref="B42:B45"/>
     <mergeCell ref="B46:B49"/>
     <mergeCell ref="B50:B53"/>
-    <mergeCell ref="B22:B25"/>
-    <mergeCell ref="B26:B29"/>
-    <mergeCell ref="B30:B33"/>
-    <mergeCell ref="B34:B37"/>
-    <mergeCell ref="B38:B41"/>
-    <mergeCell ref="C85:D85"/>
-    <mergeCell ref="C80:D80"/>
-    <mergeCell ref="C81:D81"/>
-    <mergeCell ref="C82:D82"/>
-    <mergeCell ref="C83:D83"/>
-    <mergeCell ref="C84:D84"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" r:id="rId1"/>
@@ -31262,21 +31493,21 @@
     </row>
     <row r="5" spans="1:19" ht="39" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A5" s="2"/>
-      <c r="B5" s="173" t="s">
+      <c r="B5" s="205" t="s">
         <v>258</v>
       </c>
-      <c r="C5" s="174"/>
-      <c r="D5" s="174"/>
-      <c r="E5" s="174"/>
-      <c r="F5" s="174"/>
-      <c r="G5" s="174"/>
-      <c r="H5" s="174"/>
-      <c r="I5" s="174"/>
-      <c r="J5" s="174"/>
-      <c r="K5" s="174"/>
-      <c r="L5" s="174"/>
-      <c r="M5" s="174"/>
-      <c r="N5" s="175"/>
+      <c r="C5" s="206"/>
+      <c r="D5" s="206"/>
+      <c r="E5" s="206"/>
+      <c r="F5" s="206"/>
+      <c r="G5" s="206"/>
+      <c r="H5" s="206"/>
+      <c r="I5" s="206"/>
+      <c r="J5" s="206"/>
+      <c r="K5" s="206"/>
+      <c r="L5" s="206"/>
+      <c r="M5" s="206"/>
+      <c r="N5" s="207"/>
       <c r="O5" s="5"/>
       <c r="P5" s="2"/>
       <c r="Q5" s="2"/>
@@ -31356,21 +31587,21 @@
       <c r="F9" s="16"/>
     </row>
     <row r="10" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B10" s="176" t="s">
+      <c r="B10" s="208" t="s">
         <v>260</v>
       </c>
     </row>
     <row r="11" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B11" s="176"/>
+      <c r="B11" s="208"/>
     </row>
     <row r="12" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B12" s="176"/>
+      <c r="B12" s="208"/>
     </row>
     <row r="13" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B13" s="176"/>
+      <c r="B13" s="208"/>
     </row>
     <row r="14" spans="1:19" x14ac:dyDescent="0.25">
-      <c r="B14" s="176"/>
+      <c r="B14" s="208"/>
     </row>
     <row r="21" spans="18:18" x14ac:dyDescent="0.25">
       <c r="R21" s="18"/>
@@ -31390,12 +31621,25 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <SharedWithUsers xmlns="d03ffd70-462c-4172-9015-a0cdff42c83c">
+      <UserInfo>
+        <DisplayName>Craig Stevens</DisplayName>
+        <AccountId>17</AccountId>
+        <AccountType/>
+      </UserInfo>
+      <UserInfo>
+        <DisplayName>Afzan Matloob</DisplayName>
+        <AccountId>46</AccountId>
+        <AccountType/>
+      </UserInfo>
+    </SharedWithUsers>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65f98c99-c090-489b-8346-b847c18a5011">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -31616,31 +31860,21 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <SharedWithUsers xmlns="d03ffd70-462c-4172-9015-a0cdff42c83c">
-      <UserInfo>
-        <DisplayName>Craig Stevens</DisplayName>
-        <AccountId>17</AccountId>
-        <AccountType/>
-      </UserInfo>
-      <UserInfo>
-        <DisplayName>Afzan Matloob</DisplayName>
-        <AccountId>46</AccountId>
-        <AccountType/>
-      </UserInfo>
-    </SharedWithUsers>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="65f98c99-c090-489b-8346-b847c18a5011">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7D0D882-CBE1-41A5-A59C-C48B26872275}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F627C2A1-639E-4000-94D7-FA9740411AFB}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="d03ffd70-462c-4172-9015-a0cdff42c83c"/>
+    <ds:schemaRef ds:uri="65f98c99-c090-489b-8346-b847c18a5011"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -31665,12 +31899,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F627C2A1-639E-4000-94D7-FA9740411AFB}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F7D0D882-CBE1-41A5-A59C-C48B26872275}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="d03ffd70-462c-4172-9015-a0cdff42c83c"/>
-    <ds:schemaRef ds:uri="65f98c99-c090-489b-8346-b847c18a5011"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>

</xml_diff>